<commit_message>
Add 2x DOLD 80x16S profile as drag chain holders
The two upper base_drag_chain_holder parts are replaced by DOLD
60886-Z aluminium profile 80x16S Nut 8, cut to 650 mm. The two lower
holders stay printed parts. M3 threads on top are drilled in-house.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Bestellliste.xlsx
+++ b/bom/Bestellliste.xlsx
@@ -1090,7 +1090,43 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Aluprofil I-Typ 80x16S Nut 8, 650 mm (Energieketten-Halter)</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>nein (nicht im Angebot AN2026-104489) – Art.-Nr. 60886-Z</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="3">
+        <f>0.65*28+0.5</f>
+        <v/>
+      </c>
+      <c r="F13" s="3">
+        <f>D13*E13</f>
+        <v/>
+      </c>
       <c r="G13" s="3" t="n"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ERSATZ für Druckteil base_drag_chain_holder (obere Halter :1 und :3); die 2 unteren bleiben Druckteil. Je Profil 20 × M3-Gewinde auf der Oberseite selbst bohren/schneiden (Kernloch 2,5 mm)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://www.dold-mechatronik.de/Aluminiumprofil-80x16S-I-Typ-Nut-8-schwer-22kg-m-Zuschnitt-50-6000mm</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Add igus E2i.10 drag chains to order list
X axis: E2i.10.20.028.0, 14 links (0.28 m) with E2.100.20.34PZ.A2 brackets.
Y axis: E2i.10.10.028.0, 12 links (0.24 m) with E2.100.10.34PZ.A2 brackets.
Both 2 per probe. Inserted row 92; totals shifted and re-checked.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Bestellliste.xlsx
+++ b/bom/Bestellliste.xlsx
@@ -781,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM115"/>
+  <dimension ref="A1:BM116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -3181,7 +3181,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Energieketten</t>
+          <t>Energiekette igus E2i.10.20.028.0 (X), 14 Glieder = 0,28 m, inkl. Anschlussset E2.100.20.34PZ.A2</t>
         </is>
       </c>
       <c r="B91" s="25" t="inlineStr">
@@ -3189,348 +3189,418 @@
           <t>nein</t>
         </is>
       </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>2</v>
+      </c>
+      <c r="E91">
+        <f>(14*0.49+6.48)*1.19</f>
+        <v/>
+      </c>
+      <c r="F91">
+        <f>D91*E91</f>
+        <v/>
+      </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>2 je Probe (8 im Vollausbau). igus-Preise netto: 0,49 €/Glied + 6,48 € Anschlussset, hier inkl. 19 % MwSt.; versandfertig in 24 h</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>https://www.igus.de/product/series-E2i-10?artnr=E2I.10.20.028.0</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
+          <t>Energiekette igus E2i.10.10.028.0 (Y), 12 Glieder = 0,24 m, inkl. Anschlussset E2.100.10.34PZ.A2</t>
+        </is>
+      </c>
+      <c r="B92" s="25" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>2</v>
+      </c>
+      <c r="E92">
+        <f>(12*0.47+6.2)*1.19</f>
+        <v/>
+      </c>
+      <c r="F92">
+        <f>D92*E92</f>
+        <v/>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>2 je Probe (8 im Vollausbau). Die 8 kollidierenden Doppel-Ketten im CAD wurden gelöscht. igus-Preise netto: 0,47 €/Glied + 6,20 € Anschlussset, hier inkl. 19 % MwSt.; versandfertig in 72 h</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>https://www.igus.de/product/series-E2i-10?artnr=E2i.10.10.028.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
           <t>Kabel für Endschalter</t>
         </is>
       </c>
-      <c r="B92" s="25" t="inlineStr">
+      <c r="B93" s="25" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="G92" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="17" t="inlineStr">
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="inlineStr">
         <is>
           <t>Motorkabel</t>
         </is>
       </c>
-      <c r="B93" s="25" t="inlineStr">
+      <c r="B94" s="25" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="C93" s="18" t="n"/>
-      <c r="D93" s="18" t="n"/>
-      <c r="E93" s="18" t="n"/>
-      <c r="F93" s="18" t="n"/>
-      <c r="G93" s="18" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H93" s="17" t="n"/>
-      <c r="I93" s="17" t="n"/>
-      <c r="J93" s="17" t="n"/>
-      <c r="K93" s="17" t="n"/>
-      <c r="L93" s="17" t="n"/>
-      <c r="M93" s="17" t="n"/>
-      <c r="N93" s="17" t="n"/>
-      <c r="O93" s="17" t="n"/>
-      <c r="P93" s="17" t="n"/>
-      <c r="Q93" s="17" t="n"/>
-      <c r="R93" s="17" t="n"/>
-      <c r="S93" s="17" t="n"/>
-      <c r="T93" s="17" t="n"/>
-      <c r="U93" s="17" t="n"/>
-      <c r="V93" s="17" t="n"/>
-      <c r="W93" s="17" t="n"/>
-      <c r="X93" s="17" t="n"/>
-      <c r="Y93" s="17" t="n"/>
-      <c r="Z93" s="17" t="n"/>
-      <c r="AA93" s="17" t="n"/>
-      <c r="AB93" s="17" t="n"/>
-      <c r="AC93" s="17" t="n"/>
-      <c r="AD93" s="17" t="n"/>
-      <c r="AE93" s="17" t="n"/>
-      <c r="AF93" s="17" t="n"/>
-      <c r="AG93" s="17" t="n"/>
-      <c r="AH93" s="17" t="n"/>
-      <c r="AI93" s="17" t="n"/>
-      <c r="AJ93" s="17" t="n"/>
-      <c r="AK93" s="17" t="n"/>
-      <c r="AL93" s="17" t="n"/>
-      <c r="AM93" s="17" t="n"/>
-      <c r="AN93" s="17" t="n"/>
-      <c r="AO93" s="17" t="n"/>
-      <c r="AP93" s="17" t="n"/>
-      <c r="AQ93" s="17" t="n"/>
-      <c r="AR93" s="17" t="n"/>
-      <c r="AS93" s="17" t="n"/>
-      <c r="AT93" s="17" t="n"/>
-      <c r="AU93" s="17" t="n"/>
-      <c r="AV93" s="17" t="n"/>
-      <c r="AW93" s="17" t="n"/>
-      <c r="AX93" s="17" t="n"/>
-      <c r="AY93" s="17" t="n"/>
-      <c r="AZ93" s="17" t="n"/>
-      <c r="BA93" s="17" t="n"/>
-      <c r="BB93" s="17" t="n"/>
-      <c r="BC93" s="17" t="n"/>
-      <c r="BD93" s="17" t="n"/>
-      <c r="BE93" s="17" t="n"/>
-      <c r="BF93" s="17" t="n"/>
-      <c r="BG93" s="17" t="n"/>
-      <c r="BH93" s="17" t="n"/>
-      <c r="BI93" s="17" t="n"/>
-      <c r="BJ93" s="17" t="n"/>
-      <c r="BK93" s="17" t="n"/>
-      <c r="BL93" s="17" t="n"/>
-      <c r="BM93" s="17" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t>Rahmen / Gestell (einmalig) inkl. Mwst.</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="n"/>
-      <c r="D94" s="5" t="n"/>
-      <c r="E94" s="5" t="n"/>
-      <c r="F94" s="5">
-        <f>SUM(F6:F24)</f>
-        <v/>
-      </c>
-      <c r="G94" s="3" t="n"/>
+      <c r="C94" s="18" t="n"/>
+      <c r="D94" s="18" t="n"/>
+      <c r="E94" s="18" t="n"/>
+      <c r="F94" s="18" t="n"/>
+      <c r="G94" s="18" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H94" s="17" t="n"/>
+      <c r="I94" s="17" t="n"/>
+      <c r="J94" s="17" t="n"/>
+      <c r="K94" s="17" t="n"/>
+      <c r="L94" s="17" t="n"/>
+      <c r="M94" s="17" t="n"/>
+      <c r="N94" s="17" t="n"/>
+      <c r="O94" s="17" t="n"/>
+      <c r="P94" s="17" t="n"/>
+      <c r="Q94" s="17" t="n"/>
+      <c r="R94" s="17" t="n"/>
+      <c r="S94" s="17" t="n"/>
+      <c r="T94" s="17" t="n"/>
+      <c r="U94" s="17" t="n"/>
+      <c r="V94" s="17" t="n"/>
+      <c r="W94" s="17" t="n"/>
+      <c r="X94" s="17" t="n"/>
+      <c r="Y94" s="17" t="n"/>
+      <c r="Z94" s="17" t="n"/>
+      <c r="AA94" s="17" t="n"/>
+      <c r="AB94" s="17" t="n"/>
+      <c r="AC94" s="17" t="n"/>
+      <c r="AD94" s="17" t="n"/>
+      <c r="AE94" s="17" t="n"/>
+      <c r="AF94" s="17" t="n"/>
+      <c r="AG94" s="17" t="n"/>
+      <c r="AH94" s="17" t="n"/>
+      <c r="AI94" s="17" t="n"/>
+      <c r="AJ94" s="17" t="n"/>
+      <c r="AK94" s="17" t="n"/>
+      <c r="AL94" s="17" t="n"/>
+      <c r="AM94" s="17" t="n"/>
+      <c r="AN94" s="17" t="n"/>
+      <c r="AO94" s="17" t="n"/>
+      <c r="AP94" s="17" t="n"/>
+      <c r="AQ94" s="17" t="n"/>
+      <c r="AR94" s="17" t="n"/>
+      <c r="AS94" s="17" t="n"/>
+      <c r="AT94" s="17" t="n"/>
+      <c r="AU94" s="17" t="n"/>
+      <c r="AV94" s="17" t="n"/>
+      <c r="AW94" s="17" t="n"/>
+      <c r="AX94" s="17" t="n"/>
+      <c r="AY94" s="17" t="n"/>
+      <c r="AZ94" s="17" t="n"/>
+      <c r="BA94" s="17" t="n"/>
+      <c r="BB94" s="17" t="n"/>
+      <c r="BC94" s="17" t="n"/>
+      <c r="BD94" s="17" t="n"/>
+      <c r="BE94" s="17" t="n"/>
+      <c r="BF94" s="17" t="n"/>
+      <c r="BG94" s="17" t="n"/>
+      <c r="BH94" s="17" t="n"/>
+      <c r="BI94" s="17" t="n"/>
+      <c r="BJ94" s="17" t="n"/>
+      <c r="BK94" s="17" t="n"/>
+      <c r="BL94" s="17" t="n"/>
+      <c r="BM94" s="17" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Rahmen / Gestell (einmalig) exkl. Mwst.</t>
+          <t>Rahmen / Gestell (einmalig) inkl. Mwst.</t>
         </is>
       </c>
       <c r="C95" s="5" t="n"/>
       <c r="D95" s="5" t="n"/>
       <c r="E95" s="5" t="n"/>
-      <c r="F95" s="19">
-        <f>F94/1.19</f>
+      <c r="F95" s="5">
+        <f>SUM(F6:F24)</f>
         <v/>
       </c>
       <c r="G95" s="3" t="n"/>
     </row>
     <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>Rahmen / Gestell (einmalig) exkl. Mwst.</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="n"/>
+      <c r="D96" s="5" t="n"/>
+      <c r="E96" s="5" t="n"/>
+      <c r="F96" s="19">
+        <f>F95/1.19</f>
+        <v/>
+      </c>
       <c r="G96" s="3" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="inlineStr">
-        <is>
-          <t>je weitere Probe inkl. Mwst.</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="n"/>
-      <c r="D97" s="5" t="n"/>
-      <c r="E97" s="5" t="n"/>
-      <c r="F97" s="19">
-        <f>SUM(F27:F93)</f>
-        <v/>
-      </c>
       <c r="G97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>je weitere Probe exkl. Mwst.</t>
+          <t>je weitere Probe inkl. Mwst.</t>
         </is>
       </c>
       <c r="C98" s="5" t="n"/>
       <c r="D98" s="5" t="n"/>
       <c r="E98" s="5" t="n"/>
       <c r="F98" s="19">
-        <f>F97/1.19</f>
+        <f>SUM(F27:F94)</f>
         <v/>
       </c>
       <c r="G98" s="3" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="4" t="n"/>
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>je weitere Probe exkl. Mwst.</t>
+        </is>
+      </c>
       <c r="C99" s="5" t="n"/>
       <c r="D99" s="5" t="n"/>
       <c r="E99" s="5" t="n"/>
-      <c r="F99" s="19" t="n"/>
+      <c r="F99" s="19">
+        <f>F98/1.19</f>
+        <v/>
+      </c>
       <c r="G99" s="3" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="inlineStr">
-        <is>
-          <t>Prototyp = Rahmen mit 1 x Probe inkl. Mwst.</t>
-        </is>
-      </c>
+      <c r="A100" s="4" t="n"/>
       <c r="C100" s="5" t="n"/>
       <c r="D100" s="5" t="n"/>
       <c r="E100" s="5" t="n"/>
-      <c r="F100" s="19">
-        <f>SUM(F6:F93)</f>
-        <v/>
-      </c>
-      <c r="G100" s="19" t="n"/>
+      <c r="F100" s="19" t="n"/>
+      <c r="G100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Prototyp = Rahmen mit 1 x Probe exkl. Mwst.</t>
+          <t>Prototyp = Rahmen mit 1 x Probe inkl. Mwst.</t>
         </is>
       </c>
       <c r="C101" s="5" t="n"/>
       <c r="D101" s="5" t="n"/>
       <c r="E101" s="5" t="n"/>
       <c r="F101" s="19">
-        <f>F100/1.19</f>
+        <f>SUM(F6:F94)</f>
         <v/>
       </c>
       <c r="G101" s="19" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="4" t="n"/>
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>Prototyp = Rahmen mit 1 x Probe exkl. Mwst.</t>
+        </is>
+      </c>
       <c r="C102" s="5" t="n"/>
       <c r="D102" s="5" t="n"/>
       <c r="E102" s="5" t="n"/>
-      <c r="F102" s="5" t="n"/>
-      <c r="G102" s="5" t="n"/>
+      <c r="F102" s="19">
+        <f>F101/1.19</f>
+        <v/>
+      </c>
+      <c r="G102" s="19" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="inlineStr">
-        <is>
-          <t>Vollausbau = Rahmen + 4 x Probe inkl. Mwst.</t>
-        </is>
-      </c>
+      <c r="A103" s="4" t="n"/>
       <c r="C103" s="5" t="n"/>
       <c r="D103" s="5" t="n"/>
       <c r="E103" s="5" t="n"/>
-      <c r="F103" s="19">
-        <f>F100+3*F97</f>
-        <v/>
-      </c>
-      <c r="G103" s="19" t="n"/>
+      <c r="F103" s="5" t="n"/>
+      <c r="G103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>Vollausbau = Rahmen + 4 x Probe exkl. Mwst.</t>
+          <t>Vollausbau = Rahmen + 4 x Probe inkl. Mwst.</t>
         </is>
       </c>
       <c r="C104" s="5" t="n"/>
       <c r="D104" s="5" t="n"/>
       <c r="E104" s="5" t="n"/>
       <c r="F104" s="19">
-        <f>F103/1.19</f>
+        <f>F101+3*F98</f>
         <v/>
       </c>
       <c r="G104" s="19" t="n"/>
     </row>
-    <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="6" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>Vollausbau = Rahmen + 4 x Probe exkl. Mwst.</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="n"/>
+      <c r="D105" s="5" t="n"/>
+      <c r="E105" s="5" t="n"/>
+      <c r="F105" s="19">
+        <f>F104/1.19</f>
+        <v/>
+      </c>
+      <c r="G105" s="19" t="n"/>
+    </row>
+    <row r="107" ht="15.75" customHeight="1"/>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
         <is>
           <t>Farbcode Hersteller</t>
         </is>
       </c>
-      <c r="C107" s="7" t="n"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="8" t="inlineStr">
+      <c r="C108" s="7" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
         <is>
           <t>DOLD Mechatronik: https://www.dold-mechatronik.de</t>
         </is>
       </c>
-      <c r="C108" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="13" t="inlineStr">
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="13" t="inlineStr">
         <is>
           <t>Nanotec: https://de.nanotec.com</t>
         </is>
       </c>
-      <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="16" t="inlineStr">
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="inlineStr">
         <is>
           <t>igus: https://www.igus.de</t>
         </is>
       </c>
-      <c r="C110" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="9" t="inlineStr">
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="9" t="inlineStr">
         <is>
           <t>Teleskopschienen24: https://www.teleskopschienen24.de/</t>
         </is>
       </c>
-      <c r="C111" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="12" t="inlineStr">
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="12" t="inlineStr">
         <is>
           <t>Motedis: https://www.motedis.com/</t>
         </is>
       </c>
-      <c r="C112" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="F112" s="20" t="n"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="15" t="inlineStr">
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="F113" s="20" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="15" t="inlineStr">
         <is>
           <t>Amazon: https://www.amazon.de</t>
         </is>
       </c>
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="F113" s="10" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="11" t="inlineStr">
-        <is>
-          <t>Laserteile4you: https://www.laserteile4you.de/home.html</t>
-        </is>
-      </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
+      <c r="F114" s="10" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="11" t="inlineStr">
         <is>
+          <t>Laserteile4you: https://www.laserteile4you.de/home.html</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="inlineStr">
+        <is>
           <t>StepperOnline: https://www.omc-stepperonline.com</t>
         </is>
       </c>
-      <c r="C115" s="3" t="inlineStr">
+      <c r="C116" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>

</xml_diff>

<commit_message>
Update order list: sensors, shaft holders, belts, spindle parts, slides
- Inductive end stops: M8 LJ8A3-2-Z/BX (Amazon) instead of M12 AI905,
  3 per probe as used by the firmware
- Add 4x DOLD SHF10 flange shaft holders per probe
- GT2 6 mm wheels, idlers and belt sized for X, Y and Z
  (4 + 4 per probe, 5 m belt per probe)
- Spindle drive parts set to 0 (belt drive in CAD), DOLD positions
  15, 17, 18, 24, 25 marked for removal
- Drawer slides: DOLD HS-4613-350 instead of Teleskopschienen24

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Bestellliste.xlsx
+++ b/bom/Bestellliste.xlsx
@@ -993,12 +993,12 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Teleskopauszug TS-A 514613-350mm mit Arretierung</t>
+          <t>Teleskopschienen Vollauszug 45 kg, 350 mm (1 Paar), DOLD HS-4613-350</t>
         </is>
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>nein (nicht im Angebot AN2026-104489) – Art.-Nr. HS-4613-350</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1010,16 +1010,21 @@
         <v>1</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>12.5</v>
+        <v>10.84</v>
       </c>
       <c r="F10" s="3">
         <f>D10*E10</f>
         <v/>
       </c>
       <c r="G10" s="3" t="n"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ERSATZ für Teleskopschienen24 TS-A 514613-350 (12,50 €/Paar, mit Arretierung). DOLD: 45,7 × 12,7 mm wie CAD, Arretierung nicht angegeben, Lochbild beim Einbau prüfen</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://www.teleskopschienen24.de/vollauszug-tsaa-514613-350mm</t>
+          <t>https://www.dold-mechatronik.de/Vollauszug-45kg-350mm-(1-Paar-Teleskopschienen)</t>
         </is>
       </c>
     </row>
@@ -1368,30 +1373,40 @@
       <c r="G21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Profilschienenführung, MR12, 600mm, Edelstahl</t>
         </is>
       </c>
-      <c r="B22" s="25" t="inlineStr">
-        <is>
-          <t>nein</t>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>nein (nicht im Angebot AN2026-104489) – Art.-Nr. 78553-600</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>55.12</v>
+        <v>82.2</v>
       </c>
       <c r="F22" s="3">
         <f>D22*E22</f>
         <v/>
       </c>
       <c r="G22" s="3" t="n"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ERSATZ des Motedis-Artikels MR12M-N L=600 (Art. 6111): gleiche Schiene (cpc MR12M, Edelstahl, Genauigkeit N, V0). Preis 82,20 € inkl. 19 % USt. laut DOLD-Shop (Stand 27.10.2026), sofort lieferbar</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://www.motedis.com/shop/Dynamik-Lineareinheiten/Profilschienenfuehrungen-fuer-die-Linearbewegung/Profilschienenfuehrungen/Profilschienenfuehrung-Miniatur-MR12M-N-L-%3D-600mm::6111.html</t>
+          <t>https://www.dold-mechatronik.de/Linearfuehrung-MR-12-M-Edelstahl-600mm</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1628,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>8.5</v>
@@ -1625,6 +1640,11 @@
       <c r="G30" s="3" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD); DOLD-Angebot Pos 15 streichen lassen</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1646,12 +1666,12 @@
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>Endschalter induktiv M12 x 1</t>
+          <t>Endschalter induktiv M8, LJ8A3-2-Z/BX (NPN, Schließer, 2 mm)</t>
         </is>
       </c>
       <c r="B34" s="24" t="inlineStr">
         <is>
-          <t>ja – Pos 16 AI905</t>
+          <t>nein (DOLD-Angebot Pos 16 AI905 M12 passt nicht – streichen lassen)</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1674,9 +1694,14 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ERSATZ für M12: CAD-Halter haben 8,1-mm-Bohrung. 2 je Probe (X-min und X-max), wie in der Firmware</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://www.amazon.de/Heschen-Induktiver-N%C3%A4herungsschalter-LJ12-A3-4-Z-normalerweise/dp/B071ZQ6VV6/</t>
+          <t>https://www.amazon.de/Induktive-N%C3%A4herungsschalter-LJ8-A3-2-z-BX-Normalerweise/dp/B072Q68493/</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1734,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E37" s="14">
         <f>20.09*1.19</f>
@@ -1724,6 +1749,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD)</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>https://www.igus.de/product/847</t>
@@ -1747,7 +1777,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>5.9</v>
@@ -1761,6 +1791,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD); DOLD-Angebot Pos 17 streichen lassen</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Aluminumgehaeuse-SCE12SFX</t>
@@ -1784,7 +1819,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>0.15</v>
@@ -1796,6 +1831,11 @@
       <c r="G39" s="3" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD); DOLD-Angebot Pos 18 streichen lassen</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2121,7 +2161,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E50" s="3" t="n">
         <v>8.5</v>
@@ -2135,6 +2175,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD); DOLD-Angebot Pos 24 streichen lassen</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Spielfreie-Wendelkupplung-Klemmnabenausfuehrung-JT16C-D16L23-500-600mm</t>
@@ -2158,7 +2203,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>0.5</v>
@@ -2172,6 +2217,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD); DOLD-Angebot Pos 25 streichen lassen</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Rillenkugellager-626-2RS-6x19x6mm</t>
@@ -2190,7 +2240,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
@@ -2198,6 +2248,11 @@
         </is>
       </c>
       <c r="G52" s="3" t="n"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -2216,7 +2271,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E53" s="10" t="n">
         <v>21.3</v>
@@ -2230,6 +2285,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD)</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t>https://de.nanotec.com/produkte/446-st3518m1004-a/</t>
@@ -2237,7 +2297,46 @@
       </c>
     </row>
     <row r="54">
-      <c r="G54" s="3" t="n"/>
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>Wellenhalter Flansch SHF10, D10</t>
+        </is>
+      </c>
+      <c r="B54" s="24" t="inlineStr">
+        <is>
+          <t>nein (nicht im Angebot AN2026-104489)</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F54" s="3">
+        <f>D54*E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Halter für die 2 runden X-Führungswellen je Brücke, beidseitig (CAD rod_holder_flange_d10_dold, 16 im Vollausbau)</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://www.dold-mechatronik.de/Wellenhalter-Flansch-SHF-Ausfuehrung-waehlbar</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
@@ -2356,12 +2455,12 @@
     <row r="59">
       <c r="A59" s="15" t="inlineStr">
         <is>
-          <t>Endschalter induktiv M12 x 1</t>
+          <t>Endschalter induktiv M8, LJ8A3-2-Z/BX (NPN, Schließer, 2 mm)</t>
         </is>
       </c>
       <c r="B59" s="24" t="inlineStr">
         <is>
-          <t>ja – Pos 29 AI905</t>
+          <t>nein (DOLD-Angebot Pos 29 AI905 M12 passt nicht – streichen lassen)</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -2370,7 +2469,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>6.89</v>
@@ -2384,9 +2483,14 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>ERSATZ für M12: CAD-Halter haben 8,1-mm-Bohrung. 1 je Probe (Y-max), wie in der Firmware</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>https://www.amazon.de/Heschen-Induktiver-N%C3%A4herungsschalter-LJ12-A3-4-Z-normalerweise/dp/B071ZQ6VV6/</t>
+          <t>https://www.amazon.de/Induktive-N%C3%A4herungsschalter-LJ8-A3-2-z-BX-Normalerweise/dp/B072Q68493/</t>
         </is>
       </c>
     </row>
@@ -2570,7 +2674,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E67" s="14">
         <f>20.09*1.19</f>
@@ -2585,6 +2689,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>ENTFÄLLT (Riemenantrieb statt Spindel, Teil nicht im CAD)</t>
+        </is>
+      </c>
       <c r="I67" t="inlineStr">
         <is>
           <t>https://www.igus.de/product/847</t>
@@ -2717,7 +2826,7 @@
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>Zahnriemenrad GT2 6mm, 16 Zähne</t>
+          <t>Zahnriemenrad GT2 6mm, 16 Zähne, Bohrung 5 mm (X, Y, Z)</t>
         </is>
       </c>
       <c r="B71" s="24" t="inlineStr">
@@ -2731,7 +2840,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E71" s="14" t="n">
         <v>2.9</v>
@@ -2745,6 +2854,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>ANPASSUNG: 4 je Probe = 2 × X-Motor, 1 × Y-Motor, 1 × Z-Motor. DOLD-Angebot Pos 35 nur 1 Stk → auf 16 erhöhen</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Zahnriemenrad-GT2-6mm-breit-16-Zaehne-Bohrung-500mm-H7-mit-Klemmschrauben</t>
@@ -2754,7 +2868,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>Umlenkrolle GT2 6mm, 16 Zähne</t>
+          <t>Umlenkrolle GT2 6mm, 16 Zähne, mit Kugellager, Bohrung 3 mm (X, Y, Z)</t>
         </is>
       </c>
       <c r="B72" s="24" t="inlineStr">
@@ -2762,8 +2876,13 @@
           <t>ja – Pos 36 46132</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="D72" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E72" s="14" t="n">
         <v>3.2</v>
@@ -2777,6 +2896,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>ANPASSUNG: 4 je Probe = 2 × X-Riemenspanner, 1 × Y-Riemenspanner, 1 × Z-Umlenkung (CAD zeigt 20, davon 8 doppelt gezeichnet). DOLD-Angebot Pos 36 nur 1 Stk → auf 16 erhöhen</t>
+        </is>
+      </c>
       <c r="I72" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Umlenkrolle-Zahnriemenrad-mit-Kugellager-GT2-6mm-breit-16-Zaehne-Bohrung-300mm</t>
@@ -2786,7 +2910,7 @@
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>Zahnriemen GT2, 6mm, 1m</t>
+          <t>Zahnriemen GT2, 6 mm breit, je 1 Meter (X, Y, Z)</t>
         </is>
       </c>
       <c r="B73" s="24" t="inlineStr">
@@ -2800,7 +2924,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E73" s="14" t="n">
         <v>2.5</v>
@@ -2812,6 +2936,16 @@
       <c r="G73" s="3" t="inlineStr">
         <is>
           <t>x</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>ANPASSUNG: 5 m je Probe (Bedarf 4,13 m: X 2 × 1,43 m, Y 1,02 m, Z 0,25 m; CAD zeigt Z 9 mm breit, wir nehmen 6 mm). DOLD-Angebot Pos 37 nur 1 m → auf 20 m erhöhen</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>https://www.dold-mechatronik.de/Zahnriemen-GT2-Breite-6mm-Laenge-1-Meter</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Return to open-loop drives: 14HS13-0804S + BTT TMC2130 V3.0 SPI
X, Y and Z now use the StepperOnline 14HS13-0804S (NEMA 14, 18 Ncm,
0.8 A, 34.8 mm) in place of the Nanotec ST3518M1004-A, whose product
page is gone. The CL42T-V41 closed-loop drivers are removed again and
the TMC2130 V2.0 set is replaced by 4x BTT TMC2130 V3.0 SPI per probe
from Tinytronics, added to the supplier legend.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Bestellliste.xlsx
+++ b/bom/Bestellliste.xlsx
@@ -135,7 +135,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -253,6 +253,11 @@
         <bgColor rgb="FFFCD3C1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -308,7 +313,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -366,6 +371,7 @@
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="19">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -781,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM116"/>
+  <dimension ref="A1:BM117"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -1489,9 +1495,9 @@
       <c r="G26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>Closed-Loop-Schrittmotor NEMA 14 – StepperOnline 14HS11-1004-ME1K</t>
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Schrittmotor NEMA 14 – StepperOnline 14HS13-0804S</t>
         </is>
       </c>
       <c r="B27" s="25" t="inlineStr">
@@ -1507,9 +1513,8 @@
       <c r="D27" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="14">
-        <f>28.57+6.03</f>
-        <v/>
+      <c r="E27" s="14" t="n">
+        <v>7.72</v>
       </c>
       <c r="F27" s="3">
         <f>D27*E27</f>
@@ -1522,12 +1527,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>ERSATZ für Nanotec ST3518M1004-A (offen, ohne Encoder): Closed Loop, Encoder 1000 PPR, 34,5 mm inkl. Encoder, passt ohne CAD-Änderung. Preis = 28,57 € + 6,03 € Aufpreis Lager DE; MwSt. im Warenkorb prüfen</t>
+          <t>ERSATZ für Nanotec ST3518M1004-A (Produktseite nicht mehr erreichbar, Lieferbarkeit unklar): offener Regelkreis wie Original, 1,8°, 18 Ncm, 0,8 A, 6,8 Ω, 10 mH, 35x35x34,8 mm, Welle Ø5 x 24 mm mit D-Schnitt, Litze 400 mm. Firmware: X/X2/Y/Z_CURRENT von 800 auf ca. 560–600 mA RMS senken. Passung im CAD noch prüfen (Original 36 mm lang). Preis = 7,72 € Lager China (Lager DE +2,72 €, am 27.10.2026 kein DE-Bestand); MwSt. im Warenkorb prüfen</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://www.omc-stepperonline.com/nema-14-closed-loop-stepper-motor-12-5ncm-17-73oz-in-with-magnetic-encoder-1000ppr-4000cpr-14hs11-1004-me1k</t>
+          <t>https://www.omc-stepperonline.com/de/nema-14-bipolar-1-8deg-18ncm-25-5oz-in-0-8a-5-74v-35x35x34mm-4-draehte-14hs13-0804s</t>
         </is>
       </c>
     </row>
@@ -1569,47 +1574,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>Closed-Loop-Treiber StepperOnline CL42T-V41</t>
-        </is>
-      </c>
-      <c r="B29" s="25" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" s="14">
-        <f>33.11+6.16</f>
-        <v/>
-      </c>
-      <c r="F29" s="3">
-        <f>D29*E29</f>
-        <v/>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>NEU: Closed-Loop-Treiber, ersetzt TMC2130 für diese Achse. Schalter S3 auf 5 V, Pegelwandler 3,3 V → 5 V nötig. Preis = 33,11 € + 6,16 € Aufpreis Lager DE; MwSt. prüfen</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>https://www.omc-stepperonline.com/closed-loop-stepper-driver-v4-1-0-3-0a-24-48vdc-for-nema-11-14-17-stepper-motor-cl42t-v41</t>
-        </is>
-      </c>
+      <c r="G29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -2022,52 +1987,12 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>Closed-Loop-Treiber StepperOnline CL42T-V41</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="14">
-        <f>33.11+6.16</f>
-        <v/>
-      </c>
-      <c r="F47" s="14">
-        <f>D47*E47</f>
-        <v/>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>NEU: Closed-Loop-Treiber, ersetzt TMC2130 für diese Achse. Schalter S3 auf 5 V, Pegelwandler 3,3 V → 5 V nötig. Preis = 33,11 € + 6,16 € Aufpreis Lager DE; MwSt. prüfen</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>https://www.omc-stepperonline.com/closed-loop-stepper-driver-v4-1-0-3-0a-24-48vdc-for-nema-11-14-17-stepper-motor-cl42t-v41</t>
-        </is>
-      </c>
+      <c r="G47" s="3" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>Closed-Loop-Schrittmotor NEMA 14 – StepperOnline 14HS11-1004-ME1K</t>
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Schrittmotor NEMA 14 – StepperOnline 14HS13-0804S</t>
         </is>
       </c>
       <c r="B48" s="25" t="inlineStr">
@@ -2083,9 +2008,8 @@
       <c r="D48" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E48" s="14">
-        <f>28.57+6.03</f>
-        <v/>
+      <c r="E48" s="14" t="n">
+        <v>7.72</v>
       </c>
       <c r="F48" s="14">
         <f>D48*E48</f>
@@ -2098,12 +2022,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>ERSATZ für Nanotec ST3518M1004-A (offen, ohne Encoder): Closed Loop, Encoder 1000 PPR, 34,5 mm inkl. Encoder, passt ohne CAD-Änderung. Preis = 28,57 € + 6,03 € Aufpreis Lager DE; MwSt. im Warenkorb prüfen</t>
+          <t>ERSATZ für Nanotec ST3518M1004-A (Produktseite nicht mehr erreichbar, Lieferbarkeit unklar): offener Regelkreis wie Original, 1,8°, 18 Ncm, 0,8 A, 6,8 Ω, 10 mH, 35x35x34,8 mm, Welle Ø5 x 24 mm mit D-Schnitt, Litze 400 mm. Firmware: X/X2/Y/Z_CURRENT von 800 auf ca. 560–600 mA RMS senken. Passung im CAD noch prüfen (Original 36 mm lang). Preis = 7,72 € Lager China (Lager DE +2,72 €, am 27.10.2026 kein DE-Bestand); MwSt. im Warenkorb prüfen</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://www.omc-stepperonline.com/nema-14-closed-loop-stepper-motor-12-5ncm-17-73oz-in-with-magnetic-encoder-1000ppr-4000cpr-14hs11-1004-me1k</t>
+          <t>https://www.omc-stepperonline.com/de/nema-14-bipolar-1-8deg-18ncm-25-5oz-in-0-8a-5-74v-35x35x34mm-4-draehte-14hs13-0804s</t>
         </is>
       </c>
     </row>
@@ -2701,52 +2625,12 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="13" t="inlineStr">
-        <is>
-          <t>Closed-Loop-Treiber StepperOnline CL42T-V41</t>
-        </is>
-      </c>
-      <c r="B68" s="25" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" s="14">
-        <f>33.11+6.16</f>
-        <v/>
-      </c>
-      <c r="F68" s="14">
-        <f>D68*E68</f>
-        <v/>
-      </c>
-      <c r="G68" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>NEU: Closed-Loop-Treiber, ersetzt TMC2130 für diese Achse. Schalter S3 auf 5 V, Pegelwandler 3,3 V → 5 V nötig. Preis = 33,11 € + 6,16 € Aufpreis Lager DE; MwSt. prüfen</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>https://www.omc-stepperonline.com/closed-loop-stepper-driver-v4-1-0-3-0a-24-48vdc-for-nema-11-14-17-stepper-motor-cl42t-v41</t>
-        </is>
-      </c>
+      <c r="G68" s="3" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="13" t="inlineStr">
-        <is>
-          <t>Closed-Loop-Schrittmotor NEMA 14 – StepperOnline 14HS11-1004-ME1K</t>
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>Schrittmotor NEMA 14 – StepperOnline 14HS13-0804S</t>
         </is>
       </c>
       <c r="B69" s="25" t="inlineStr">
@@ -2762,9 +2646,8 @@
       <c r="D69" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E69" s="14">
-        <f>28.57+6.03</f>
-        <v/>
+      <c r="E69" s="14" t="n">
+        <v>7.72</v>
       </c>
       <c r="F69" s="14">
         <f>D69*E69</f>
@@ -2777,12 +2660,12 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>ERSATZ für Nanotec ST3518M1004-A (offen, ohne Encoder): Closed Loop, Encoder 1000 PPR, 34,5 mm inkl. Encoder, passt ohne CAD-Änderung. Preis = 28,57 € + 6,03 € Aufpreis Lager DE; MwSt. im Warenkorb prüfen</t>
+          <t>ERSATZ für Nanotec ST3518M1004-A (Produktseite nicht mehr erreichbar, Lieferbarkeit unklar): offener Regelkreis wie Original, 1,8°, 18 Ncm, 0,8 A, 6,8 Ω, 10 mH, 35x35x34,8 mm, Welle Ø5 x 24 mm mit D-Schnitt, Litze 400 mm. Firmware: X/X2/Y/Z_CURRENT von 800 auf ca. 560–600 mA RMS senken. Passung im CAD noch prüfen (Original 36 mm lang). Preis = 7,72 € Lager China (Lager DE +2,72 €, am 27.10.2026 kein DE-Bestand); MwSt. im Warenkorb prüfen</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://www.omc-stepperonline.com/nema-14-closed-loop-stepper-motor-12-5ncm-17-73oz-in-with-magnetic-encoder-1000ppr-4000cpr-14hs11-1004-me1k</t>
+          <t>https://www.omc-stepperonline.com/de/nema-14-bipolar-1-8deg-18ncm-25-5oz-in-0-8a-5-74v-35x35x34mm-4-draehte-14hs13-0804s</t>
         </is>
       </c>
     </row>
@@ -3187,9 +3070,9 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="15" t="inlineStr">
-        <is>
-          <t>4 x TMC2130 V2.0 Motortreiber</t>
+      <c r="A86" s="29" t="inlineStr">
+        <is>
+          <t>BTT TMC2130 V3.0 SPI Schrittmotortreiber</t>
         </is>
       </c>
       <c r="B86" s="25" t="inlineStr">
@@ -3203,10 +3086,10 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E86" s="10" t="n">
-        <v>33.99</v>
+        <v>8.75</v>
       </c>
       <c r="F86" s="3">
         <f>D86*E86</f>
@@ -3219,12 +3102,12 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>ANPASSUNG: X/Y/Z laufen über CL42T-V41 – TMC2130 werden dafür nicht mehr gebraucht; Menge prüfen</t>
+          <t>ERSATZ für 4 x TMC2130 V2.0 (PoPprint-Set, Amazon): gleicher Chip, aktuelles BTT-Modul in SPI-Ausführung. 4 je Probe (X, X2, Y, Z), 16 im Vollausbau. Auf der SKR die SPI-Jumper setzen. Preis = 8,75 € inkl. MwSt. bei Tinytronics (NL), 50+ auf Lager am 27.10.2026; bei BIQU ist die SPI-Variante ausverkauft, bei 3DJake nicht mehr gelistet</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://www.amazon.de/PoPprint-SPI-Motortreiber-K%C3%BChlk%C3%B6rper-Verwendung-Goldablagerungstechnologie/dp/B07Q9JKK23/</t>
+          <t>https://www.tinytronics.nl/nl/mechanica-en-actuatoren/motoraansturingen-en-drivers/stappen-motoraansturingen-en-drivers/bigtreetech-tmc2130-v3.0-stappenmotordriver-module-spi</t>
         </is>
       </c>
     </row>
@@ -3740,6 +3623,18 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" s="29" t="inlineStr">
+        <is>
+          <t>Tinytronics: https://www.tinytronics.nl</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0.3937007874015748" bottom="0.3937007874015748" header="0" footer="0"/>
   <headerFooter>

</xml_diff>

<commit_message>
Order SKR V1.4 Turbo and TMC2130 drivers from Roboter-Bausatz
The "Smoothieboard ohne Stepper Treiber" row linked to a PoPprint SKR V1.3,
which is no longer available; it is replaced by the BTT SKR V1.4 Turbo.
Board and BTT TMC2130 V3.0 SPI drivers now come from Roboter-Bausatz.de
to bundle the order; Roboter-Bausatz replaces Tinytronics in the legend.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Bestellliste.xlsx
+++ b/bom/Bestellliste.xlsx
@@ -135,7 +135,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -258,6 +258,11 @@
         <fgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9BC2E6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -313,7 +318,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -372,6 +377,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="19">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -3033,9 +3039,9 @@
       <c r="G84" s="3" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="15" t="inlineStr">
-        <is>
-          <t>Smoothieboard ohne Stepper Treiber</t>
+      <c r="A85" s="30" t="inlineStr">
+        <is>
+          <t>BIGTREETECH SKR V1.4 Turbo Mainboard (ohne Schrittmotortreiber)</t>
         </is>
       </c>
       <c r="B85" s="25" t="inlineStr">
@@ -3052,7 +3058,7 @@
         <v>1</v>
       </c>
       <c r="E85" s="10" t="n">
-        <v>25.99</v>
+        <v>49.95</v>
       </c>
       <c r="F85" s="3">
         <f>D85*E85</f>
@@ -3063,14 +3069,19 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>ERSATZ für SKR V1.3 (in der SCHUTZWERK-BOM als „Smoothieboard ohne Stepper Treiber“ bezeichnet, Amazon-Link führt auf PoPprint SKR V1.3, derzeit nicht verfügbar). LPC1769, 120 MHz, 5 steckbare Treiberplätze, TMC2130 per SPI. Firmware: MOTHERBOARD BOARD_BTT_SKR_V1_4_TURBO, PlatformIO-Umgebung LPC1769. Preis = 49,95 € inkl. MwSt. bis 4 Stück, sofort lieferbar (27.10.2026). Roboter-Bausatz RBS13645</t>
+        </is>
+      </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://www.amazon.de/gp/product/B07P73VWHK/</t>
+          <t>https://www.roboter-bausatz.de/p/btt-skr-1.4-turbo-32-bit-mainboard</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="29" t="inlineStr">
+      <c r="A86" s="30" t="inlineStr">
         <is>
           <t>BTT TMC2130 V3.0 SPI Schrittmotortreiber</t>
         </is>
@@ -3089,7 +3100,7 @@
         <v>4</v>
       </c>
       <c r="E86" s="10" t="n">
-        <v>8.75</v>
+        <v>13.65</v>
       </c>
       <c r="F86" s="3">
         <f>D86*E86</f>
@@ -3102,12 +3113,12 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>ERSATZ für 4 x TMC2130 V2.0 (PoPprint-Set, Amazon): gleicher Chip, aktuelles BTT-Modul in SPI-Ausführung. 4 je Probe (X, X2, Y, Z), 16 im Vollausbau. Auf der SKR die SPI-Jumper setzen. Preis = 8,75 € inkl. MwSt. bei Tinytronics (NL), 50+ auf Lager am 27.10.2026; bei BIQU ist die SPI-Variante ausverkauft, bei 3DJake nicht mehr gelistet</t>
+          <t>ERSATZ für 4 x TMC2130 V2.0 (PoPprint-Set, Amazon): gleicher Chip, aktuelles BTT-Modul in SPI-Ausführung. 4 je Probe (X, X2, Y, Z), 16 im Vollausbau. Auf der SKR die SPI-Jumper setzen. Preis = 13,65 € inkl. MwSt. bei 5–19 Stück (bis 4: 13,97 €, ab 20: 12,99 €), sofort lieferbar (27.10.2026), Roboter-Bausatz RBS18267. Zusammen mit dem Board bei einem Händler bestellt; bei Tinytronics (NL) 8,75 €/Stück, bei BIQU SPI-Variante ausverkauft</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://www.tinytronics.nl/nl/mechanica-en-actuatoren/motoraansturingen-en-drivers/stappen-motoraansturingen-en-drivers/bigtreetech-tmc2130-v3.0-stappenmotordriver-module-spi</t>
+          <t>https://www.roboter-bausatz.de/p/btt-tmc2130-v3.0-spi-schrittmotortreiber</t>
         </is>
       </c>
     </row>
@@ -3624,9 +3635,9 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="29" t="inlineStr">
-        <is>
-          <t>Tinytronics: https://www.tinytronics.nl</t>
+      <c r="A117" s="30" t="inlineStr">
+        <is>
+          <t>Roboter-Bausatz: https://www.roboter-bausatz.de</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add central Mean Well PSU and USB microscope to order list
One Mean Well SDR-240-24 DIN-rail supply from DOLD now powers all four
probes instead of one Kingled 200 W supply per probe. It is counted once:
the frame total includes it and the per-probe total excludes it.

Also adds a Toolcraft USB microscope per probe (Voelkner) with its
supplier in the legend.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Bestellliste.xlsx
+++ b/bom/Bestellliste.xlsx
@@ -135,7 +135,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -263,6 +263,11 @@
         <fgColor rgb="FF9BC2E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -318,7 +323,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -378,6 +383,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="19">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -793,7 +799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM117"/>
+  <dimension ref="A1:BM119"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -2951,139 +2957,139 @@
       </c>
     </row>
     <row r="79">
-      <c r="G79" s="3" t="n"/>
-    </row>
-    <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="6" t="inlineStr">
+      <c r="A79" s="31" t="inlineStr">
+        <is>
+          <t>USB-Mikroskop Toolcraft 2 MP, 20–200× (Ø33 × 110 mm)</t>
+        </is>
+      </c>
+      <c r="B79" s="25" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>57.41</v>
+      </c>
+      <c r="F79" s="3">
+        <f>D79*E79</f>
+        <v/>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>ANPASSUNG: 1 je Probe (4 im Vollausbau), voelkner Art.-Nr. D929041 (= Conrad 1713197). 57,41 € ab 3 Stück, Einzelpreis 57,99 €. Die Original-Halter y_camera_holder klemmen Ø42 mm, das Toolcraft hat Ø33 mm → je Mikroskop eine gedruckte, geschlitzte PETG-Adapterhülse Ø33/Ø42 (4,5 mm Wand). Linux/UVC und MJPEG sind vom Händler nicht angegeben: erstes Gerät mit v4l2-ctl --list-formats-ext prüfen.</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>https://www.voelkner.de/products/1177903/TOOLCRAFT-USB-Mikroskop-2-Megapixel-Digitale-Vergroesserung-max.-200-x.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="G80" s="3" t="n"/>
+    </row>
+    <row r="81" ht="15.75" customHeight="1">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t>Z-Schlitten</t>
         </is>
       </c>
-      <c r="C80" s="7" t="n"/>
-      <c r="G80" s="3" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="8" t="inlineStr">
+      <c r="C81" s="7" t="n"/>
+      <c r="G81" s="3" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
         <is>
           <t>Profilschienenführung, MR12, 150mm, Edelstahl</t>
         </is>
       </c>
-      <c r="B81" s="24" t="inlineStr">
+      <c r="B82" s="24" t="inlineStr">
         <is>
           <t>ja – Pos 40 78553-150</t>
         </is>
       </c>
-      <c r="C81" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E81" s="10" t="n">
-        <v>20.55</v>
-      </c>
-      <c r="F81" s="3">
-        <f>D81*E81</f>
-        <v/>
-      </c>
-      <c r="G81" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>https://www.dold-mechatronik.de/Linearfuehrung-MR-12-M-Edelstahl-150mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Probespitze</t>
-        </is>
-      </c>
-      <c r="B82" s="25" t="inlineStr">
-        <is>
-          <t>nein</t>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
       <c r="D82" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E82" s="10" t="inlineStr">
+      <c r="E82" s="10" t="n">
+        <v>20.55</v>
+      </c>
+      <c r="F82" s="3">
+        <f>D82*E82</f>
+        <v/>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>https://www.dold-mechatronik.de/Linearfuehrung-MR-12-M-Edelstahl-150mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Probespitze</t>
+        </is>
+      </c>
+      <c r="B83" s="25" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="10" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="G82" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="E83" s="10" t="n"/>
-      <c r="G83" s="3" t="n"/>
-    </row>
-    <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="6" t="inlineStr">
-        <is>
-          <t>Elektronik</t>
-        </is>
-      </c>
-      <c r="C84" s="7" t="n"/>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
       <c r="E84" s="10" t="n"/>
       <c r="G84" s="3" t="n"/>
     </row>
-    <row r="85">
-      <c r="A85" s="30" t="inlineStr">
-        <is>
-          <t>BIGTREETECH SKR V1.4 Turbo Mainboard (ohne Schrittmotortreiber)</t>
-        </is>
-      </c>
-      <c r="B85" s="25" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="C85" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E85" s="10" t="n">
-        <v>49.95</v>
-      </c>
-      <c r="F85" s="3">
-        <f>D85*E85</f>
-        <v/>
-      </c>
-      <c r="G85" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>ERSATZ für SKR V1.3 (in der SCHUTZWERK-BOM als „Smoothieboard ohne Stepper Treiber“ bezeichnet, Amazon-Link führt auf PoPprint SKR V1.3, derzeit nicht verfügbar). LPC1769, 120 MHz, 5 steckbare Treiberplätze, TMC2130 per SPI. Firmware: MOTHERBOARD BOARD_BTT_SKR_V1_4_TURBO, PlatformIO-Umgebung LPC1769. Preis = 49,95 € inkl. MwSt. bis 4 Stück, sofort lieferbar (27.10.2026). Roboter-Bausatz RBS13645</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>https://www.roboter-bausatz.de/p/btt-skr-1.4-turbo-32-bit-mainboard</t>
-        </is>
-      </c>
+    <row r="85" ht="15.75" customHeight="1">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>Elektronik</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="n"/>
+      <c r="E85" s="10" t="n"/>
+      <c r="G85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="30" t="inlineStr">
         <is>
-          <t>BTT TMC2130 V3.0 SPI Schrittmotortreiber</t>
+          <t>BIGTREETECH SKR V1.4 Turbo Mainboard (ohne Schrittmotortreiber)</t>
         </is>
       </c>
       <c r="B86" s="25" t="inlineStr">
@@ -3097,10 +3103,10 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E86" s="10" t="n">
-        <v>13.65</v>
+        <v>49.95</v>
       </c>
       <c r="F86" s="3">
         <f>D86*E86</f>
@@ -3113,19 +3119,19 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>ERSATZ für 4 x TMC2130 V2.0 (PoPprint-Set, Amazon): gleicher Chip, aktuelles BTT-Modul in SPI-Ausführung. 4 je Probe (X, X2, Y, Z), 16 im Vollausbau. Auf der SKR die SPI-Jumper setzen. Preis = 13,65 € inkl. MwSt. bei 5–19 Stück (bis 4: 13,97 €, ab 20: 12,99 €), sofort lieferbar (27.10.2026), Roboter-Bausatz RBS18267. Zusammen mit dem Board bei einem Händler bestellt; bei Tinytronics (NL) 8,75 €/Stück, bei BIQU SPI-Variante ausverkauft</t>
+          <t>ERSATZ für SKR V1.3 (in der SCHUTZWERK-BOM als „Smoothieboard ohne Stepper Treiber“ bezeichnet, Amazon-Link führt auf PoPprint SKR V1.3, derzeit nicht verfügbar). LPC1769, 120 MHz, 5 steckbare Treiberplätze, TMC2130 per SPI. Firmware: MOTHERBOARD BOARD_BTT_SKR_V1_4_TURBO, PlatformIO-Umgebung LPC1769. Preis = 49,95 € inkl. MwSt. bis 4 Stück, sofort lieferbar (27.10.2026). Roboter-Bausatz RBS13645</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://www.roboter-bausatz.de/p/btt-tmc2130-v3.0-spi-schrittmotortreiber</t>
+          <t>https://www.roboter-bausatz.de/p/btt-skr-1.4-turbo-32-bit-mainboard</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="15" t="inlineStr">
-        <is>
-          <t>Schaltnetzteil 24V, 8,4A, 200W</t>
+      <c r="A87" s="30" t="inlineStr">
+        <is>
+          <t>BTT TMC2130 V3.0 SPI Schrittmotortreiber</t>
         </is>
       </c>
       <c r="B87" s="25" t="inlineStr">
@@ -3139,10 +3145,10 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E87" s="3" t="n">
-        <v>37.9</v>
+        <v>4</v>
+      </c>
+      <c r="E87" s="10" t="n">
+        <v>13.65</v>
       </c>
       <c r="F87" s="3">
         <f>D87*E87</f>
@@ -3153,33 +3159,59 @@
           <t>x</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>ERSATZ für 4 x TMC2130 V2.0 (PoPprint-Set, Amazon): gleicher Chip, aktuelles BTT-Modul in SPI-Ausführung. 4 je Probe (X, X2, Y, Z), 16 im Vollausbau. Auf der SKR die SPI-Jumper setzen. Preis = 13,65 € inkl. MwSt. bei 5–19 Stück (bis 4: 13,97 €, ab 20: 12,99 €), sofort lieferbar (27.10.2026), Roboter-Bausatz RBS18267. Zusammen mit dem Board bei einem Händler bestellt; bei Tinytronics (NL) 8,75 €/Stück, bei BIQU SPI-Variante ausverkauft</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://www.amazon.de/Kingled-Netzteil-Switching-wasserdicht-kompatibel/dp/B01JOTURAK/</t>
+          <t>https://www.roboter-bausatz.de/p/btt-tmc2130-v3.0-spi-schrittmotortreiber</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Schukokabel</t>
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>Schaltnetzteil Mean Well SDR-240-24, Hutschiene, 24 V / 10 A / 240 W</t>
         </is>
       </c>
       <c r="B88" s="25" t="inlineStr">
         <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="G88" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
+          <t>nein (nicht im Angebot AN2026-104489) – Art.-Nr. SNT MW-SDR240-24</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="F88" s="3">
+        <f>D88*E88</f>
+        <v/>
+      </c>
+      <c r="G88" s="3" t="n"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>ANPASSUNG: 1 zentrales Netzteil für alle 4 Probes statt 1 je Probe (SCHUTZWERK: Kingled 24 V / 200 W je Probe). ERSATZ für Kingled: Mean Well Industrieausführung mit PFC, berührgeschützte Klemmen. Bedarf ca. 150 W im ungünstigsten Fall (16 Motoren ≤ 110 W, 4 Boards ≈ 10 W, Licht ca. 20–30 W). Verteilung auf die 4 SKR-Boards je Board abgesichert; 230-V-Seite durch Elektrofachkraft. Einmalige Position: in „Rahmen / Gestell (einmalig)“ enthalten, nicht in „je weitere Probe“. Preis = 84,79 € inkl. MwSt., sofort verfügbar (27.10.2026)</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>https://www.dold-mechatronik.de/Switching-power-supply-DIN-rail-240-W-24-V-10-A</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Kabel Probe</t>
+          <t>Schukokabel</t>
         </is>
       </c>
       <c r="B89" s="25" t="inlineStr">
@@ -3196,7 +3228,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Gehäuse für Elektronik</t>
+          <t>Kabel Probe</t>
         </is>
       </c>
       <c r="B90" s="25" t="inlineStr">
@@ -3204,12 +3236,16 @@
           <t>nein</t>
         </is>
       </c>
-      <c r="G90" s="3" t="n"/>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Energiekette igus E2i.10.20.028.0 (X), 14 Glieder = 0,28 m, inkl. Anschlussset E2.100.20.34PZ.A2</t>
+          <t>Gehäuse für Elektronik</t>
         </is>
       </c>
       <c r="B91" s="25" t="inlineStr">
@@ -3217,42 +3253,12 @@
           <t>nein</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D91" t="n">
-        <v>2</v>
-      </c>
-      <c r="E91">
-        <f>(14*0.49+6.48)*1.19</f>
-        <v/>
-      </c>
-      <c r="F91">
-        <f>D91*E91</f>
-        <v/>
-      </c>
-      <c r="G91" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>2 je Probe (8 im Vollausbau). igus-Preise netto: 0,49 €/Glied + 6,48 € Anschlussset, hier inkl. 19 % MwSt.; versandfertig in 24 h</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>https://www.igus.de/product/series-E2i-10?artnr=E2I.10.20.028.0</t>
-        </is>
-      </c>
+      <c r="G91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Energiekette igus E2i.10.10.028.0 (Y), 12 Glieder = 0,24 m, inkl. Anschlussset E2.100.10.34PZ.A2</t>
+          <t>Energiekette igus E2i.10.20.028.0 (X), 14 Glieder = 0,28 m, inkl. Anschlussset E2.100.20.34PZ.A2</t>
         </is>
       </c>
       <c r="B92" s="25" t="inlineStr">
@@ -3269,7 +3275,7 @@
         <v>2</v>
       </c>
       <c r="E92">
-        <f>(12*0.47+6.2)*1.19</f>
+        <f>(14*0.49+6.48)*1.19</f>
         <v/>
       </c>
       <c r="F92">
@@ -3283,364 +3289,419 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>2 je Probe (8 im Vollausbau). Die 8 kollidierenden Doppel-Ketten im CAD wurden gelöscht. igus-Preise netto: 0,47 €/Glied + 6,20 € Anschlussset, hier inkl. 19 % MwSt.; versandfertig in 72 h</t>
+          <t>2 je Probe (8 im Vollausbau). igus-Preise netto: 0,49 €/Glied + 6,48 € Anschlussset, hier inkl. 19 % MwSt.; versandfertig in 24 h</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://www.igus.de/product/series-E2i-10?artnr=E2i.10.10.028.0</t>
+          <t>https://www.igus.de/product/series-E2i-10?artnr=E2I.10.20.028.0</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
+          <t>Energiekette igus E2i.10.10.028.0 (Y), 12 Glieder = 0,24 m, inkl. Anschlussset E2.100.10.34PZ.A2</t>
+        </is>
+      </c>
+      <c r="B93" s="25" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>2</v>
+      </c>
+      <c r="E93">
+        <f>(12*0.47+6.2)*1.19</f>
+        <v/>
+      </c>
+      <c r="F93">
+        <f>D93*E93</f>
+        <v/>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>2 je Probe (8 im Vollausbau). Die 8 kollidierenden Doppel-Ketten im CAD wurden gelöscht. igus-Preise netto: 0,47 €/Glied + 6,20 € Anschlussset, hier inkl. 19 % MwSt.; versandfertig in 72 h</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>https://www.igus.de/product/series-E2i-10?artnr=E2i.10.10.028.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
           <t>Kabel für Endschalter</t>
         </is>
       </c>
-      <c r="B93" s="25" t="inlineStr">
+      <c r="B94" s="25" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="G93" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="17" t="inlineStr">
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="inlineStr">
         <is>
           <t>Motorkabel</t>
         </is>
       </c>
-      <c r="B94" s="25" t="inlineStr">
+      <c r="B95" s="25" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="C94" s="18" t="n"/>
-      <c r="D94" s="18" t="n"/>
-      <c r="E94" s="18" t="n"/>
-      <c r="F94" s="18" t="n"/>
-      <c r="G94" s="18" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H94" s="17" t="n"/>
-      <c r="I94" s="17" t="n"/>
-      <c r="J94" s="17" t="n"/>
-      <c r="K94" s="17" t="n"/>
-      <c r="L94" s="17" t="n"/>
-      <c r="M94" s="17" t="n"/>
-      <c r="N94" s="17" t="n"/>
-      <c r="O94" s="17" t="n"/>
-      <c r="P94" s="17" t="n"/>
-      <c r="Q94" s="17" t="n"/>
-      <c r="R94" s="17" t="n"/>
-      <c r="S94" s="17" t="n"/>
-      <c r="T94" s="17" t="n"/>
-      <c r="U94" s="17" t="n"/>
-      <c r="V94" s="17" t="n"/>
-      <c r="W94" s="17" t="n"/>
-      <c r="X94" s="17" t="n"/>
-      <c r="Y94" s="17" t="n"/>
-      <c r="Z94" s="17" t="n"/>
-      <c r="AA94" s="17" t="n"/>
-      <c r="AB94" s="17" t="n"/>
-      <c r="AC94" s="17" t="n"/>
-      <c r="AD94" s="17" t="n"/>
-      <c r="AE94" s="17" t="n"/>
-      <c r="AF94" s="17" t="n"/>
-      <c r="AG94" s="17" t="n"/>
-      <c r="AH94" s="17" t="n"/>
-      <c r="AI94" s="17" t="n"/>
-      <c r="AJ94" s="17" t="n"/>
-      <c r="AK94" s="17" t="n"/>
-      <c r="AL94" s="17" t="n"/>
-      <c r="AM94" s="17" t="n"/>
-      <c r="AN94" s="17" t="n"/>
-      <c r="AO94" s="17" t="n"/>
-      <c r="AP94" s="17" t="n"/>
-      <c r="AQ94" s="17" t="n"/>
-      <c r="AR94" s="17" t="n"/>
-      <c r="AS94" s="17" t="n"/>
-      <c r="AT94" s="17" t="n"/>
-      <c r="AU94" s="17" t="n"/>
-      <c r="AV94" s="17" t="n"/>
-      <c r="AW94" s="17" t="n"/>
-      <c r="AX94" s="17" t="n"/>
-      <c r="AY94" s="17" t="n"/>
-      <c r="AZ94" s="17" t="n"/>
-      <c r="BA94" s="17" t="n"/>
-      <c r="BB94" s="17" t="n"/>
-      <c r="BC94" s="17" t="n"/>
-      <c r="BD94" s="17" t="n"/>
-      <c r="BE94" s="17" t="n"/>
-      <c r="BF94" s="17" t="n"/>
-      <c r="BG94" s="17" t="n"/>
-      <c r="BH94" s="17" t="n"/>
-      <c r="BI94" s="17" t="n"/>
-      <c r="BJ94" s="17" t="n"/>
-      <c r="BK94" s="17" t="n"/>
-      <c r="BL94" s="17" t="n"/>
-      <c r="BM94" s="17" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="4" t="inlineStr">
-        <is>
-          <t>Rahmen / Gestell (einmalig) inkl. Mwst.</t>
-        </is>
-      </c>
-      <c r="C95" s="5" t="n"/>
-      <c r="D95" s="5" t="n"/>
-      <c r="E95" s="5" t="n"/>
-      <c r="F95" s="5">
-        <f>SUM(F6:F24)</f>
-        <v/>
-      </c>
-      <c r="G95" s="3" t="n"/>
+      <c r="C95" s="18" t="n"/>
+      <c r="D95" s="18" t="n"/>
+      <c r="E95" s="18" t="n"/>
+      <c r="F95" s="18" t="n"/>
+      <c r="G95" s="18" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H95" s="17" t="n"/>
+      <c r="I95" s="17" t="n"/>
+      <c r="J95" s="17" t="n"/>
+      <c r="K95" s="17" t="n"/>
+      <c r="L95" s="17" t="n"/>
+      <c r="M95" s="17" t="n"/>
+      <c r="N95" s="17" t="n"/>
+      <c r="O95" s="17" t="n"/>
+      <c r="P95" s="17" t="n"/>
+      <c r="Q95" s="17" t="n"/>
+      <c r="R95" s="17" t="n"/>
+      <c r="S95" s="17" t="n"/>
+      <c r="T95" s="17" t="n"/>
+      <c r="U95" s="17" t="n"/>
+      <c r="V95" s="17" t="n"/>
+      <c r="W95" s="17" t="n"/>
+      <c r="X95" s="17" t="n"/>
+      <c r="Y95" s="17" t="n"/>
+      <c r="Z95" s="17" t="n"/>
+      <c r="AA95" s="17" t="n"/>
+      <c r="AB95" s="17" t="n"/>
+      <c r="AC95" s="17" t="n"/>
+      <c r="AD95" s="17" t="n"/>
+      <c r="AE95" s="17" t="n"/>
+      <c r="AF95" s="17" t="n"/>
+      <c r="AG95" s="17" t="n"/>
+      <c r="AH95" s="17" t="n"/>
+      <c r="AI95" s="17" t="n"/>
+      <c r="AJ95" s="17" t="n"/>
+      <c r="AK95" s="17" t="n"/>
+      <c r="AL95" s="17" t="n"/>
+      <c r="AM95" s="17" t="n"/>
+      <c r="AN95" s="17" t="n"/>
+      <c r="AO95" s="17" t="n"/>
+      <c r="AP95" s="17" t="n"/>
+      <c r="AQ95" s="17" t="n"/>
+      <c r="AR95" s="17" t="n"/>
+      <c r="AS95" s="17" t="n"/>
+      <c r="AT95" s="17" t="n"/>
+      <c r="AU95" s="17" t="n"/>
+      <c r="AV95" s="17" t="n"/>
+      <c r="AW95" s="17" t="n"/>
+      <c r="AX95" s="17" t="n"/>
+      <c r="AY95" s="17" t="n"/>
+      <c r="AZ95" s="17" t="n"/>
+      <c r="BA95" s="17" t="n"/>
+      <c r="BB95" s="17" t="n"/>
+      <c r="BC95" s="17" t="n"/>
+      <c r="BD95" s="17" t="n"/>
+      <c r="BE95" s="17" t="n"/>
+      <c r="BF95" s="17" t="n"/>
+      <c r="BG95" s="17" t="n"/>
+      <c r="BH95" s="17" t="n"/>
+      <c r="BI95" s="17" t="n"/>
+      <c r="BJ95" s="17" t="n"/>
+      <c r="BK95" s="17" t="n"/>
+      <c r="BL95" s="17" t="n"/>
+      <c r="BM95" s="17" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>Rahmen / Gestell (einmalig) exkl. Mwst.</t>
+          <t>Rahmen / Gestell (einmalig) inkl. Mwst.</t>
         </is>
       </c>
       <c r="C96" s="5" t="n"/>
       <c r="D96" s="5" t="n"/>
       <c r="E96" s="5" t="n"/>
-      <c r="F96" s="19">
-        <f>F95/1.19</f>
+      <c r="F96" s="5">
+        <f>SUM(F6:F24)+F88</f>
         <v/>
       </c>
       <c r="G96" s="3" t="n"/>
     </row>
     <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>Rahmen / Gestell (einmalig) exkl. Mwst.</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="n"/>
+      <c r="D97" s="5" t="n"/>
+      <c r="E97" s="5" t="n"/>
+      <c r="F97" s="19">
+        <f>F96/1.19</f>
+        <v/>
+      </c>
       <c r="G97" s="3" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="4" t="inlineStr">
-        <is>
-          <t>je weitere Probe inkl. Mwst.</t>
-        </is>
-      </c>
-      <c r="C98" s="5" t="n"/>
-      <c r="D98" s="5" t="n"/>
-      <c r="E98" s="5" t="n"/>
-      <c r="F98" s="19">
-        <f>SUM(F27:F94)</f>
-        <v/>
-      </c>
       <c r="G98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>je weitere Probe exkl. Mwst.</t>
+          <t>je weitere Probe inkl. Mwst.</t>
         </is>
       </c>
       <c r="C99" s="5" t="n"/>
       <c r="D99" s="5" t="n"/>
       <c r="E99" s="5" t="n"/>
       <c r="F99" s="19">
-        <f>F98/1.19</f>
+        <f>SUM(F27:F95)-F88</f>
         <v/>
       </c>
       <c r="G99" s="3" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="n"/>
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>je weitere Probe exkl. Mwst.</t>
+        </is>
+      </c>
       <c r="C100" s="5" t="n"/>
       <c r="D100" s="5" t="n"/>
       <c r="E100" s="5" t="n"/>
-      <c r="F100" s="19" t="n"/>
+      <c r="F100" s="19">
+        <f>F99/1.19</f>
+        <v/>
+      </c>
       <c r="G100" s="3" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="4" t="inlineStr">
-        <is>
-          <t>Prototyp = Rahmen mit 1 x Probe inkl. Mwst.</t>
-        </is>
-      </c>
+      <c r="A101" s="4" t="n"/>
       <c r="C101" s="5" t="n"/>
       <c r="D101" s="5" t="n"/>
       <c r="E101" s="5" t="n"/>
-      <c r="F101" s="19">
-        <f>SUM(F6:F94)</f>
-        <v/>
-      </c>
-      <c r="G101" s="19" t="n"/>
+      <c r="F101" s="19" t="n"/>
+      <c r="G101" s="3" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>Prototyp = Rahmen mit 1 x Probe exkl. Mwst.</t>
+          <t>Prototyp = Rahmen mit 1 x Probe inkl. Mwst.</t>
         </is>
       </c>
       <c r="C102" s="5" t="n"/>
       <c r="D102" s="5" t="n"/>
       <c r="E102" s="5" t="n"/>
       <c r="F102" s="19">
-        <f>F101/1.19</f>
+        <f>SUM(F6:F95)</f>
         <v/>
       </c>
       <c r="G102" s="19" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="n"/>
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>Prototyp = Rahmen mit 1 x Probe exkl. Mwst.</t>
+        </is>
+      </c>
       <c r="C103" s="5" t="n"/>
       <c r="D103" s="5" t="n"/>
       <c r="E103" s="5" t="n"/>
-      <c r="F103" s="5" t="n"/>
-      <c r="G103" s="5" t="n"/>
+      <c r="F103" s="19">
+        <f>F102/1.19</f>
+        <v/>
+      </c>
+      <c r="G103" s="19" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="4" t="inlineStr">
-        <is>
-          <t>Vollausbau = Rahmen + 4 x Probe inkl. Mwst.</t>
-        </is>
-      </c>
+      <c r="A104" s="4" t="n"/>
       <c r="C104" s="5" t="n"/>
       <c r="D104" s="5" t="n"/>
       <c r="E104" s="5" t="n"/>
-      <c r="F104" s="19">
-        <f>F101+3*F98</f>
-        <v/>
-      </c>
-      <c r="G104" s="19" t="n"/>
+      <c r="F104" s="5" t="n"/>
+      <c r="G104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>Vollausbau = Rahmen + 4 x Probe exkl. Mwst.</t>
+          <t>Vollausbau = Rahmen + 4 x Probe inkl. Mwst.</t>
         </is>
       </c>
       <c r="C105" s="5" t="n"/>
       <c r="D105" s="5" t="n"/>
       <c r="E105" s="5" t="n"/>
       <c r="F105" s="19">
-        <f>F104/1.19</f>
+        <f>F102+3*F99</f>
         <v/>
       </c>
       <c r="G105" s="19" t="n"/>
     </row>
-    <row r="107" ht="15.75" customHeight="1"/>
-    <row r="108">
-      <c r="A108" s="6" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>Vollausbau = Rahmen + 4 x Probe exkl. Mwst.</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="n"/>
+      <c r="D106" s="5" t="n"/>
+      <c r="E106" s="5" t="n"/>
+      <c r="F106" s="19">
+        <f>F105/1.19</f>
+        <v/>
+      </c>
+      <c r="G106" s="19" t="n"/>
+    </row>
+    <row r="108" ht="15.75" customHeight="1"/>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
         <is>
           <t>Farbcode Hersteller</t>
         </is>
       </c>
-      <c r="C108" s="7" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="8" t="inlineStr">
+      <c r="C109" s="7" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
         <is>
           <t>DOLD Mechatronik: https://www.dold-mechatronik.de</t>
         </is>
       </c>
-      <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="13" t="inlineStr">
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="13" t="inlineStr">
         <is>
           <t>Nanotec: https://de.nanotec.com</t>
         </is>
       </c>
-      <c r="C110" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="16" t="inlineStr">
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="16" t="inlineStr">
         <is>
           <t>igus: https://www.igus.de</t>
         </is>
       </c>
-      <c r="C111" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="9" t="inlineStr">
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="9" t="inlineStr">
         <is>
           <t>Teleskopschienen24: https://www.teleskopschienen24.de/</t>
         </is>
       </c>
-      <c r="C112" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="12" t="inlineStr">
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="12" t="inlineStr">
         <is>
           <t>Motedis: https://www.motedis.com/</t>
         </is>
       </c>
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="F113" s="20" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="15" t="inlineStr">
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="F114" s="20" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="15" t="inlineStr">
         <is>
           <t>Amazon: https://www.amazon.de</t>
         </is>
       </c>
-      <c r="C114" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="F114" s="10" t="n"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="11" t="inlineStr">
-        <is>
-          <t>Laserteile4you: https://www.laserteile4you.de/home.html</t>
-        </is>
-      </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
+      <c r="F115" s="10" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
+          <t>Laserteile4you: https://www.laserteile4you.de/home.html</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="inlineStr">
+        <is>
           <t>StepperOnline: https://www.omc-stepperonline.com</t>
         </is>
       </c>
-      <c r="C116" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="30" t="inlineStr">
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="30" t="inlineStr">
         <is>
           <t>Roboter-Bausatz: https://www.roboter-bausatz.de</t>
         </is>
       </c>
-      <c r="C117" s="3" t="inlineStr">
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="31" t="inlineStr">
+        <is>
+          <t>Voelkner: https://www.voelkner.de</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>

</xml_diff>

<commit_message>
Add DOLD order list, status column and per-shop sheet
- New bom/Dold Bestellung.xlsx: all DOLD items with full-build
  quantity (4 probes) and link, without prices
- Bestellliste: notes column removed, offer highlighting removed,
  new status column (identifiziert, bestellt, geliefert, verbaut)
- New sheet "nach Hersteller" grouping all parts by shop, linked
  to the main sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/Bestellliste.xlsx
+++ b/bom/Bestellliste.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1560" yWindow="1560" windowWidth="27630" windowHeight="17745" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Bestellliste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="nach Hersteller" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,14 +26,27 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -42,16 +55,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
+        <fgColor rgb="FFFFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -63,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -85,9 +112,24 @@
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -450,8 +492,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H102"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H103"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -460,16 +502,17 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Bestellliste ProBoter</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -503,12 +546,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Anmerkung</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
           <t>Link</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -519,8 +562,7 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -533,8 +575,7 @@
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -558,14 +599,14 @@
         <v/>
       </c>
       <c r="F6" s="4" t="n"/>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 1)</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Gelenkfuss-Reihe-10-PA-Gewindestange-mit-Kugel-10mm-M6x20-Schluesselweite-10-Teller-40mm-mit-Anti-Slip-Platte-40-d385</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -591,14 +632,14 @@
         <v/>
       </c>
       <c r="F7" s="4" t="n"/>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 2)</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Winkel-30-I-Typ-Nut-6-inkl-Befestigungssatz-und-Abdeckkappe</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -624,18 +665,18 @@
         <v/>
       </c>
       <c r="F8" s="4" t="n"/>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 3)</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Buegelgriff-100mm-mit-Befestigungsbohrungen</t>
         </is>
       </c>
-    </row>
-    <row r="9">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Teleskopschienen Vollauszug 45 kg, 350 mm (1 Paar), DOLD HS-4613-350</t>
@@ -657,18 +698,18 @@
         <v/>
       </c>
       <c r="F9" s="4" t="n"/>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für Teleskopschienen24 TS-A 514613-350 (12,50 €/Paar, mit Arretierung). DOLD: 45,7 × 12,7 mm wie CAD, Arretierung nicht angegeben, Lochbild beim Einbau prüfen</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Vollauszug-45kg-350mm-(1-Paar-Teleskopschienen)</t>
         </is>
       </c>
-    </row>
-    <row r="10">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Aluprofil I-Typ 80x16S Nut 8, 650 mm (Energieketten-Halter)</t>
@@ -691,14 +732,14 @@
         <v/>
       </c>
       <c r="F10" s="4" t="n"/>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für Druckteil base_drag_chain_holder (obere Halter :1 und :3); die 2 unteren bleiben Druckteil. Je Profil 20 × M3-Gewinde auf der Oberseite selbst bohren/schneiden (Kernloch 2,5 mm)</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Aluminiumprofil-80x16S-I-Typ-Nut-8-schwer-22kg-m-Zuschnitt-50-6000mm</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -724,18 +765,18 @@
         <v/>
       </c>
       <c r="F11" s="4" t="n"/>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Balken für X-Führung (DOLD-Angebot Pos 7)</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Aluminiumprofil-30x60L-I-Typ-Nut-6-ZUSCHNITT-bis-1200-mm-1700-EUR-m-030-EUR-pro-Schnitt</t>
         </is>
       </c>
-    </row>
-    <row r="12">
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Aluprofil I-Typ 30x30x350</t>
@@ -757,14 +798,14 @@
         <v/>
       </c>
       <c r="F12" s="4" t="n"/>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>4 x Senkrechte Streben + 4 x kurze Querstreben + 2 x Schublade quer (DOLD-Angebot Pos 8)</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Aluminiumprofil-30x30L-I-Typ-Nut-6-ZUSCHNITT-bis-1200-mm-850-EUR-m-025-EUR-pro-Schnitt</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -790,14 +831,14 @@
         <v/>
       </c>
       <c r="F13" s="4" t="n"/>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Längsstreben horizontal (DOLD-Angebot Pos 9)</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Aluminiumprofil-30x30L-I-Typ-Nut-6-ZUSCHNITT-bis-1200-mm-850-EUR-m-025-EUR-pro-Schnitt</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -823,14 +864,14 @@
         <v/>
       </c>
       <c r="F14" s="4" t="n"/>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Schublade längs (DOLD-Angebot Pos 10)</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Aluminiumprofil-30x30L-I-Typ-Nut-6-ZUSCHNITT-bis-1200-mm-850-EUR-m-025-EUR-pro-Schnitt</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -852,8 +893,7 @@
         <v/>
       </c>
       <c r="F15" s="4" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -877,10 +917,14 @@
         <v/>
       </c>
       <c r="F16" s="4" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="7" t="n"/>
-    </row>
-    <row r="17">
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Profilschienenführung, MR12, 600mm, Edelstahl</t>
@@ -902,18 +946,18 @@
         <v/>
       </c>
       <c r="F17" s="4" t="n"/>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ des Motedis-Artikels MR12M-N L=600 (Art. 6111): gleiche Schiene (cpc MR12M, Edelstahl, Genauigkeit N, V0). Preis 82,20 € inkl. 19 % USt. laut DOLD-Shop (Stand 27.10.2026), sofort lieferbar</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Linearfuehrung-MR-12-M-Edelstahl-600mm</t>
         </is>
       </c>
-    </row>
-    <row r="18">
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Übersichtskamera ELP 8MP USB-Kameramodul IMX179, 75° ohne Verzerrung</t>
@@ -935,14 +979,14 @@
         <v/>
       </c>
       <c r="F18" s="4" t="n"/>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für die stationäre Übersichtskamera (Modell im Original unbekannt; vorher ELP-USBFHD01M-H100, nur auf Anfrage bei ELP). 1 je Gestell. Amazon ASIN B07FXBW81G, Verkäufer ELPUSBCAMERA. 3264×2448 MJPEG 15 fps, UVC, M12-Objektiv. Bei ca. 356 mm Abstand ca. 550 mm Bildbreite (≈0,17 mm/px). ANPASSUNG prüfen: camera_holder hat Tasche 38×33 mm und M2-Raster 28×28 mm; Platine ist 38×38 mm, Lochbild nicht belegt.</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>https://www.amazon.de/dp/B07FXBW81G</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -968,14 +1012,14 @@
         <v/>
       </c>
       <c r="F19" s="4" t="n"/>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>aus Blatt BOM_2 übernommen; einzeln, sonst Teil des Gelenkfuß-Sets</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Teller-40-fuer-Gelenkstellfuss-Kugel-10mm-Kunststoff</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -986,8 +1030,7 @@
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1000,10 +1043,9 @@
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="4" t="n"/>
-    </row>
-    <row r="22">
+      <c r="G21" s="4" t="n"/>
+    </row>
+    <row r="22" ht="105" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Schrittmotor NEMA 14 – StepperOnline 14HS13-0804S</t>
@@ -1029,18 +1071,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für Nanotec ST3518M1004-A (Produktseite nicht mehr erreichbar, Lieferbarkeit unklar): offener Regelkreis wie Original, 1,8°, 18 Ncm, 0,8 A, 6,8 Ω, 10 mH, 35x35x34,8 mm, Welle Ø5 x 24 mm mit D-Schnitt, Litze 400 mm. Firmware: X/X2/Y/Z_CURRENT von 800 auf ca. 560–600 mA RMS senken. Passung im CAD noch prüfen (Original 36 mm lang). Preis = 7,72 € Lager China (Lager DE +2,72 €, am 27.10.2026 kein DE-Bestand); MwSt. im Warenkorb prüfen</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>https://www.omc-stepperonline.com/de/nema-14-bipolar-1-8deg-18ncm-25-5oz-in-0-8a-5-74v-35x35x34mm-4-draehte-14hs13-0804s</t>
         </is>
       </c>
-    </row>
-    <row r="23">
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Endschalter induktiv M8, LJ8A3-2-Z/BX (NPN, Schließer, 2 mm)</t>
@@ -1066,14 +1108,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für M12: CAD-Halter haben 8,1-mm-Bohrung. 2 je Probe (X-min und X-max), wie in der Firmware</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>https://www.amazon.de/Induktive-N%C3%A4herungsschalter-LJ8-A3-2-z-BX-Normalerweise/dp/B072Q68493/</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1084,8 +1126,7 @@
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1098,8 +1139,7 @@
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1127,14 +1167,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 19)</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>https://www.motedis.com/shop/Dynamik-Lineareinheiten/Profilschienenfuehrungen-fuer-die-Linearbewegung/Profilschienenfuehrungen/Fuehrungswagen-Miniatur-MR12MN-SS-V0-N::6097.html</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1164,14 +1204,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 21)</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Aluminiumprofil-40x16S-I-Typ-Nut-8-ZUSCHNITT-bis-1200-mm-1050-EUR-m-025-EUR-pro-Schnitt</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1201,10 +1241,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="7" t="n"/>
-    </row>
-    <row r="29">
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="105" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Schrittmotor NEMA 14 – StepperOnline 14HS13-0804S</t>
@@ -1230,18 +1274,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für Nanotec ST3518M1004-A (Produktseite nicht mehr erreichbar, Lieferbarkeit unklar): offener Regelkreis wie Original, 1,8°, 18 Ncm, 0,8 A, 6,8 Ω, 10 mH, 35x35x34,8 mm, Welle Ø5 x 24 mm mit D-Schnitt, Litze 400 mm. Firmware: X/X2/Y/Z_CURRENT von 800 auf ca. 560–600 mA RMS senken. Passung im CAD noch prüfen (Original 36 mm lang). Preis = 7,72 € Lager China (Lager DE +2,72 €, am 27.10.2026 kein DE-Bestand); MwSt. im Warenkorb prüfen</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>https://www.omc-stepperonline.com/de/nema-14-bipolar-1-8deg-18ncm-25-5oz-in-0-8a-5-74v-35x35x34mm-4-draehte-14hs13-0804s</t>
         </is>
       </c>
-    </row>
-    <row r="30">
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Wellenhalter Flansch SHF10, D10</t>
@@ -1267,14 +1311,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Halter für die 2 runden X-Führungswellen je Brücke, beidseitig (CAD rod_holder_flange_d10_dold, 16 im Vollausbau)</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Wellenhalter-Flansch-SHF-Ausfuehrung-waehlbar</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1304,18 +1348,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 26)</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Praezisionswelle-10mm-h6-geschliffen-gehaertet-450mm-mit-Gewindebohrungen-M5x20</t>
         </is>
       </c>
-    </row>
-    <row r="32">
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Endschalter induktiv M8, LJ8A3-2-Z/BX (NPN, Schließer, 2 mm)</t>
@@ -1341,14 +1385,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für M12: CAD-Halter haben 8,1-mm-Bohrung. 1 je Probe (Y-max), wie in der Firmware</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>https://www.amazon.de/Induktive-N%C3%A4herungsschalter-LJ8-A3-2-z-BX-Normalerweise/dp/B072Q68493/</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1359,8 +1403,7 @@
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1373,8 +1416,7 @@
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
-      <c r="G34" s="3" t="n"/>
-      <c r="H34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1402,14 +1444,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 32)</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Vollkunststofflager-RJMP-01-10-DryLinZ-von-igusZ</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1439,18 +1481,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 33)</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-472-Form-I-Sicherungsring-fuer-Bohrungen-Stahl-blank-I22</t>
         </is>
       </c>
-    </row>
-    <row r="37">
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="105" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Schrittmotor NEMA 14 – StepperOnline 14HS13-0804S</t>
@@ -1476,18 +1518,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für Nanotec ST3518M1004-A (Produktseite nicht mehr erreichbar, Lieferbarkeit unklar): offener Regelkreis wie Original, 1,8°, 18 Ncm, 0,8 A, 6,8 Ω, 10 mH, 35x35x34,8 mm, Welle Ø5 x 24 mm mit D-Schnitt, Litze 400 mm. Firmware: X/X2/Y/Z_CURRENT von 800 auf ca. 560–600 mA RMS senken. Passung im CAD noch prüfen (Original 36 mm lang). Preis = 7,72 € Lager China (Lager DE +2,72 €, am 27.10.2026 kein DE-Bestand); MwSt. im Warenkorb prüfen</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>https://www.omc-stepperonline.com/de/nema-14-bipolar-1-8deg-18ncm-25-5oz-in-0-8a-5-74v-35x35x34mm-4-draehte-14hs13-0804s</t>
         </is>
       </c>
-    </row>
-    <row r="38">
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Zahnriemenrad GT2 6mm, 16 Zähne, Bohrung 5 mm (X, Y, Z)</t>
@@ -1513,18 +1555,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>ANPASSUNG: 4 je Probe = 2 × X-Motor, 1 × Y-Motor, 1 × Z-Motor. DOLD-Angebot Pos 35 nur 1 Stk → auf 16 erhöhen (DOLD-Angebot Pos 35)</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Zahnriemenrad-GT2-6mm-breit-16-Zaehne-Bohrung-500mm-H7-mit-Klemmschrauben</t>
         </is>
       </c>
-    </row>
-    <row r="39">
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Umlenkrolle GT2 6mm, 16 Zähne, mit Kugellager, Bohrung 3 mm (X, Y, Z)</t>
@@ -1550,18 +1592,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>ANPASSUNG: 4 je Probe = 2 × X-Riemenspanner, 1 × Y-Riemenspanner, 1 × Z-Umlenkung (CAD zeigt 20, davon 8 doppelt gezeichnet). DOLD-Angebot Pos 36 nur 1 Stk → auf 16 erhöhen (DOLD-Angebot Pos 36)</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Umlenkrolle-Zahnriemenrad-mit-Kugellager-GT2-6mm-breit-16-Zaehne-Bohrung-300mm</t>
         </is>
       </c>
-    </row>
-    <row r="40">
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="45" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t>Zahnriemen GT2, 6 mm breit, je 1 Meter (X, Y, Z)</t>
@@ -1587,14 +1629,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>ANPASSUNG: 5 m je Probe (Bedarf 4,13 m: X 2 × 1,43 m, Y 1,02 m, Z 0,25 m; CAD zeigt Z 9 mm breit, wir nehmen 6 mm). DOLD-Angebot Pos 37 nur 1 m → auf 20 m erhöhen (DOLD-Angebot Pos 37)</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Zahnriemen-GT2-Breite-6mm-Laenge-1-Meter</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1624,14 +1666,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 38)</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>https://www.motedis.com/shop/Dynamik-Lineareinheiten/Profilschienenfuehrungen-fuer-die-Linearbewegung/Profilschienenfuehrungen/Fuehrungswagen-Miniatur-MR12MN-SS-V0-N::6097.html</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1661,14 +1703,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G42" s="3" t="n"/>
-      <c r="H42" s="4" t="inlineStr">
+      <c r="G42" s="4" t="inlineStr">
         <is>
           <t>https://www.amazon.de/gp/product/B07PX8ZFXN/ref=ox_sc_act_title_2?smid=AS8JK4HNTE2NO&amp;psc=1</t>
         </is>
       </c>
-    </row>
-    <row r="43">
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="90" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t>USB-Mikroskop Toolcraft 2 MP, 20–200× (Ø33 × 110 mm)</t>
@@ -1694,14 +1740,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>ANPASSUNG: 1 je Probe (4 im Vollausbau), voelkner Art.-Nr. D929041 (= Conrad 1713197). 57,41 € ab 3 Stück, Einzelpreis 57,99 €. Die Original-Halter y_camera_holder klemmen Ø42 mm, das Toolcraft hat Ø33 mm → je Mikroskop eine gedruckte, geschlitzte PETG-Adapterhülse Ø33/Ø42 (4,5 mm Wand). Linux/UVC und MJPEG sind vom Händler nicht angegeben: erstes Gerät mit v4l2-ctl --list-formats-ext prüfen.</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>https://www.voelkner.de/products/1177903/TOOLCRAFT-USB-Mikroskop-2-Megapixel-Digitale-Vergroesserung-max.-200-x.html</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1712,8 +1758,7 @@
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="n"/>
-      <c r="G44" s="3" t="n"/>
-      <c r="H44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -1726,8 +1771,7 @@
       <c r="D45" s="4" t="n"/>
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="4" t="n"/>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -1755,14 +1799,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 40)</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Linearfuehrung-MR-12-M-Edelstahl-150mm</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1790,8 +1834,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G47" s="3" t="n"/>
-      <c r="H47" s="7" t="n"/>
+      <c r="G47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -1800,8 +1843,7 @@
       <c r="D48" s="4" t="n"/>
       <c r="E48" s="4" t="n"/>
       <c r="F48" s="4" t="n"/>
-      <c r="G48" s="3" t="n"/>
-      <c r="H48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -1814,10 +1856,9 @@
       <c r="D49" s="4" t="n"/>
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="4" t="n"/>
-      <c r="G49" s="3" t="n"/>
-      <c r="H49" s="4" t="n"/>
-    </row>
-    <row r="50">
+      <c r="G49" s="4" t="n"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
       <c r="A50" s="3" t="inlineStr">
         <is>
           <t>BIGTREETECH SKR V1.4 Turbo Mainboard (ohne Schrittmotortreiber)</t>
@@ -1843,18 +1884,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für SKR V1.3 (in der SCHUTZWERK-BOM als „Smoothieboard ohne Stepper Treiber“ bezeichnet, Amazon-Link führt auf PoPprint SKR V1.3, derzeit nicht verfügbar). LPC1769, 120 MHz, 5 steckbare Treiberplätze, TMC2130 per SPI. Firmware: MOTHERBOARD BOARD_BTT_SKR_V1_4_TURBO, PlatformIO-Umgebung LPC1769. Preis = 49,95 € inkl. MwSt. bis 4 Stück, sofort lieferbar (27.10.2026). Roboter-Bausatz RBS13645</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="G50" s="4" t="inlineStr">
         <is>
           <t>https://www.roboter-bausatz.de/p/btt-skr-1.4-turbo-32-bit-mainboard</t>
         </is>
       </c>
-    </row>
-    <row r="51">
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="90" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>BTT TMC2130 V3.0 SPI Schrittmotortreiber</t>
@@ -1880,18 +1921,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>ERSATZ für 4 x TMC2130 V2.0 (PoPprint-Set, Amazon): gleicher Chip, aktuelles BTT-Modul in SPI-Ausführung. 4 je Probe (X, X2, Y, Z), 16 im Vollausbau. Auf der SKR die SPI-Jumper setzen. Preis = 13,65 € inkl. MwSt. bei 5–19 Stück (bis 4: 13,97 €, ab 20: 12,99 €), sofort lieferbar (27.10.2026), Roboter-Bausatz RBS18267. Zusammen mit dem Board bei einem Händler bestellt; bei Tinytronics (NL) 8,75 €/Stück, bei BIQU SPI-Variante ausverkauft</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
+      <c r="G51" s="4" t="inlineStr">
         <is>
           <t>https://www.roboter-bausatz.de/p/btt-tmc2130-v3.0-spi-schrittmotortreiber</t>
         </is>
       </c>
-    </row>
-    <row r="52">
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="120" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
           <t>Schaltnetzteil Mean Well SDR-240-24, Hutschiene, 24 V / 10 A / 240 W</t>
@@ -1913,14 +1954,14 @@
         <v/>
       </c>
       <c r="F52" s="4" t="n"/>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>ANPASSUNG: 1 zentrales Netzteil für alle 4 Probes statt 1 je Probe (SCHUTZWERK: Kingled 24 V / 200 W je Probe). ERSATZ für Kingled: Mean Well Industrieausführung mit PFC, berührgeschützte Klemmen. Bedarf ca. 150 W im ungünstigsten Fall (16 Motoren ≤ 110 W, 4 Boards ≈ 10 W, Licht ca. 20–30 W). Verteilung auf die 4 SKR-Boards je Board abgesichert; 230-V-Seite durch Elektrofachkraft. Einmalige Position: in „Rahmen / Gestell (einmalig)“ enthalten, nicht in „je weitere Probe“. Preis = 84,79 € inkl. MwSt., sofort verfügbar (27.10.2026)</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
+      <c r="G52" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Switching-power-supply-DIN-rail-240-W-24-V-10-A</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -1942,8 +1983,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G53" s="3" t="n"/>
-      <c r="H53" s="7" t="n"/>
+      <c r="G53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -1963,8 +2003,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G54" s="3" t="n"/>
-      <c r="H54" s="7" t="n"/>
+      <c r="G54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -1980,10 +2019,9 @@
         <v/>
       </c>
       <c r="F55" s="4" t="n"/>
-      <c r="G55" s="3" t="n"/>
-      <c r="H55" s="7" t="n"/>
-    </row>
-    <row r="56">
+      <c r="G55" s="7" t="n"/>
+    </row>
+    <row r="56" ht="30" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Energiekette igus E2i.10.20.028.0 (X), 14 Glieder = 0,28 m, inkl. Anschlussset E2.100.20.34PZ.A2</t>
@@ -2010,18 +2048,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>2 je Probe (8 im Vollausbau). igus-Preise netto: 0,49 €/Glied + 6,48 € Anschlussset, hier inkl. 19 % MwSt.; versandfertig in 24 h</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>https://www.igus.de/product/series-E2i-10?artnr=E2I.10.20.028.0</t>
         </is>
       </c>
-    </row>
-    <row r="57">
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="45" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Energiekette igus E2i.10.10.028.0 (Y), 12 Glieder = 0,24 m, inkl. Anschlussset E2.100.10.34PZ.A2</t>
@@ -2048,14 +2086,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>2 je Probe (8 im Vollausbau). Die 8 kollidierenden Doppel-Ketten im CAD wurden gelöscht. igus-Preise netto: 0,47 €/Glied + 6,20 € Anschlussset, hier inkl. 19 % MwSt.; versandfertig in 72 h</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>https://www.igus.de/product/series-E2i-10?artnr=E2i.10.10.028.0</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2077,8 +2115,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G58" s="3" t="n"/>
-      <c r="H58" s="7" t="n"/>
+      <c r="G58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -2098,8 +2135,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G59" s="3" t="n"/>
-      <c r="H59" s="7" t="n"/>
+      <c r="G59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -2123,14 +2159,14 @@
         <v/>
       </c>
       <c r="F60" s="4" t="n"/>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>aus Blatt BOM_2 übernommen</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr">
+      <c r="G60" s="4" t="inlineStr">
         <is>
           <t>https://www.amazon.de/Anker-Datenhub-Ultrabooks-weiteren-kompatiblen/dp/B00Y211AFM/</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2141,8 +2177,7 @@
       <c r="D61" s="4" t="n"/>
       <c r="E61" s="4" t="n"/>
       <c r="F61" s="4" t="n"/>
-      <c r="G61" s="3" t="n"/>
-      <c r="H61" s="4" t="n"/>
+      <c r="G61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -2155,8 +2190,7 @@
       <c r="D62" s="4" t="n"/>
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="n"/>
-      <c r="G62" s="3" t="n"/>
-      <c r="H62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -2178,14 +2212,14 @@
         <v/>
       </c>
       <c r="F63" s="4" t="n"/>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>CAD 52 + Reserve 6; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr">
+      <c r="G63" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2209,14 +2243,14 @@
         <v/>
       </c>
       <c r="F64" s="4" t="n"/>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>CAD 60 + Reserve 6; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H64" s="4" t="inlineStr">
+      <c r="G64" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2240,14 +2274,14 @@
         <v/>
       </c>
       <c r="F65" s="4" t="n"/>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
-          <t>CAD 8 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr">
+      <c r="G65" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2271,14 +2305,14 @@
         <v/>
       </c>
       <c r="F66" s="4" t="n"/>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>CAD 4 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H66" s="4" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2302,14 +2336,14 @@
         <v/>
       </c>
       <c r="F67" s="4" t="n"/>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>CAD 20 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
+      <c r="G67" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2333,14 +2367,14 @@
         <v/>
       </c>
       <c r="F68" s="4" t="n"/>
-      <c r="G68" s="3" t="inlineStr">
-        <is>
-          <t>CAD 32 + Reserve 4; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2364,14 +2398,14 @@
         <v/>
       </c>
       <c r="F69" s="4" t="n"/>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>CAD 4 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
+      <c r="G69" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2395,14 +2429,14 @@
         <v/>
       </c>
       <c r="F70" s="4" t="n"/>
-      <c r="G70" s="3" t="inlineStr">
-        <is>
-          <t>CAD 8 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H70" s="4" t="inlineStr">
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2426,14 +2460,14 @@
         <v/>
       </c>
       <c r="F71" s="4" t="n"/>
-      <c r="G71" s="3" t="inlineStr">
-        <is>
-          <t>CAD 1 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H71" s="4" t="inlineStr">
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2457,14 +2491,14 @@
         <v/>
       </c>
       <c r="F72" s="4" t="n"/>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>CAD 12 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H72" s="4" t="inlineStr">
+      <c r="G72" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2488,14 +2522,14 @@
         <v/>
       </c>
       <c r="F73" s="4" t="n"/>
-      <c r="G73" s="3" t="inlineStr">
-        <is>
-          <t>CAD 28 + Reserve 3; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
+      <c r="G73" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2519,14 +2553,14 @@
         <v/>
       </c>
       <c r="F74" s="4" t="n"/>
-      <c r="G74" s="3" t="inlineStr">
-        <is>
-          <t>CAD 32 + Reserve 4; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H74" s="4" t="inlineStr">
+      <c r="G74" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2550,14 +2584,14 @@
         <v/>
       </c>
       <c r="F75" s="4" t="n"/>
-      <c r="G75" s="3" t="inlineStr">
-        <is>
-          <t>CAD 4 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
+      <c r="G75" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-912-Zylinderschraube-mit-Innensechskant-8.8-verzinkt</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2581,14 +2615,14 @@
         <v/>
       </c>
       <c r="F76" s="4" t="n"/>
-      <c r="G76" s="3" t="inlineStr">
-        <is>
-          <t>CAD 32 + Reserve 4; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H76" s="4" t="inlineStr">
+      <c r="G76" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2612,14 +2646,14 @@
         <v/>
       </c>
       <c r="F77" s="4" t="n"/>
-      <c r="G77" s="3" t="inlineStr">
-        <is>
-          <t>CAD 16 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
+      <c r="G77" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2643,14 +2677,14 @@
         <v/>
       </c>
       <c r="F78" s="4" t="n"/>
-      <c r="G78" s="3" t="inlineStr">
-        <is>
-          <t>CAD 6 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H78" s="4" t="inlineStr">
+      <c r="G78" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2674,14 +2708,14 @@
         <v/>
       </c>
       <c r="F79" s="4" t="n"/>
-      <c r="G79" s="3" t="inlineStr">
-        <is>
-          <t>CAD 22 + Reserve 3; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
+      <c r="G79" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-7991-Senkschraube-mit-Innensechskant,-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2705,14 +2739,14 @@
         <v/>
       </c>
       <c r="F80" s="4" t="n"/>
-      <c r="G80" s="3" t="inlineStr">
-        <is>
-          <t>CAD 8 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H80" s="4" t="inlineStr">
+      <c r="G80" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-933-A2-Edelstahl-Sechskantschraube-mit-Gewinde-bis-Kopf.-Ausfuehrung-waehlbar</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2738,14 +2772,14 @@
         <v/>
       </c>
       <c r="F81" s="4" t="n"/>
-      <c r="G81" s="3" t="inlineStr">
-        <is>
-          <t>CAD 36 + Reserve 4</t>
-        </is>
-      </c>
-      <c r="H81" s="4" t="inlineStr">
+      <c r="G81" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-934-Sechskantmutter-.8-verzinkt-M4x07</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2771,14 +2805,14 @@
         <v/>
       </c>
       <c r="F82" s="4" t="n"/>
-      <c r="G82" s="3" t="inlineStr">
-        <is>
-          <t>CAD 48 + Reserve 5</t>
-        </is>
-      </c>
-      <c r="H82" s="4" t="inlineStr">
+      <c r="G82" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-934-Sechskantmutter-.8-verzinkt-M4x07</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2804,14 +2838,14 @@
         <v/>
       </c>
       <c r="F83" s="4" t="n"/>
-      <c r="G83" s="3" t="inlineStr">
-        <is>
-          <t>CAD 48 + Reserve 5</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
+      <c r="G83" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Sechskantmutter-DIN-934-ISO-4032-M8-Edelstahl-A2</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2835,18 +2869,18 @@
         <v/>
       </c>
       <c r="F84" s="4" t="n"/>
-      <c r="G84" s="3" t="inlineStr">
-        <is>
-          <t>CAD 8 + Reserve 2; Stückpreis je Größe im Shop wählen</t>
-        </is>
-      </c>
-      <c r="H84" s="4" t="inlineStr">
+      <c r="G84" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Hohe-Raendelmutter-Material-und-Groesse-waehlbar-NEU</t>
         </is>
       </c>
-    </row>
-    <row r="85">
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="30" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
           <t>DIN 562 Vierkantmutter flach M3</t>
@@ -2862,14 +2896,9 @@
         <v/>
       </c>
       <c r="F85" s="4" t="n"/>
-      <c r="G85" s="3" t="inlineStr">
-        <is>
-          <t>CAD 8 + Reserve 2; bei DOLD nicht erhältlich (DIN 557 zu dick für die Druckteil-Taschen), extern beschaffen</t>
-        </is>
-      </c>
-      <c r="H85" s="7" t="n"/>
-    </row>
-    <row r="86">
+      <c r="G85" s="7" t="n"/>
+    </row>
+    <row r="86" ht="30" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
           <t>DIN 562 Vierkantmutter flach M4</t>
@@ -2885,14 +2914,9 @@
         <v/>
       </c>
       <c r="F86" s="4" t="n"/>
-      <c r="G86" s="3" t="inlineStr">
-        <is>
-          <t>CAD 12 + Reserve 2; bei DOLD nicht erhältlich (DIN 557 zu dick für die Druckteil-Taschen), extern beschaffen</t>
-        </is>
-      </c>
-      <c r="H86" s="7" t="n"/>
-    </row>
-    <row r="87">
+      <c r="G86" s="7" t="n"/>
+    </row>
+    <row r="87" ht="30" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
           <t>Nutenstein Nut6, M5</t>
@@ -2914,18 +2938,18 @@
         <v/>
       </c>
       <c r="F87" s="4" t="n"/>
-      <c r="G87" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 6) Menge aus SCHUTZWERK-BOM, nicht im CAD gezeichnet.</t>
-        </is>
-      </c>
-      <c r="H87" s="4" t="inlineStr">
+      <c r="G87" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Nutenstein-mit-Steg-I-Typ-Nut-6-Gewindedurchmesser-M5</t>
         </is>
       </c>
-    </row>
-    <row r="88">
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="30" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
           <t>Nutenstein Nut6, M3</t>
@@ -2947,18 +2971,18 @@
         <v/>
       </c>
       <c r="F88" s="4" t="n"/>
-      <c r="G88" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 12) Menge aus SCHUTZWERK-BOM, nicht im CAD gezeichnet.</t>
-        </is>
-      </c>
-      <c r="H88" s="4" t="inlineStr">
+      <c r="G88" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/Nutenstein-mit-Steg-I-Typ-Nut-6-Gewindedurchmesser-M3</t>
         </is>
       </c>
-    </row>
-    <row r="89">
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="30" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
           <t>Unterlegscheiben M5</t>
@@ -2980,14 +3004,14 @@
         <v/>
       </c>
       <c r="F89" s="4" t="n"/>
-      <c r="G89" s="3" t="inlineStr">
-        <is>
-          <t>(DOLD-Angebot Pos 27) 4 je Probe = 16 im Vollausbau. Menge aus SCHUTZWERK-BOM, nicht im CAD gezeichnet.</t>
-        </is>
-      </c>
-      <c r="H89" s="4" t="inlineStr">
+      <c r="G89" s="4" t="inlineStr">
         <is>
           <t>https://www.dold-mechatronik.de/DIN-125-Form-A-Unterlegscheibe-Stahl-verzinkt-d53mm-D10mm</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>identifiziert</t>
         </is>
       </c>
     </row>
@@ -2998,8 +3022,7 @@
       <c r="D90" s="4" t="n"/>
       <c r="E90" s="4" t="n"/>
       <c r="F90" s="4" t="n"/>
-      <c r="G90" s="3" t="n"/>
-      <c r="H90" s="4" t="n"/>
+      <c r="G90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n"/>
@@ -3008,8 +3031,7 @@
       <c r="D91" s="4" t="n"/>
       <c r="E91" s="4" t="n"/>
       <c r="F91" s="4" t="n"/>
-      <c r="G91" s="3" t="n"/>
-      <c r="H91" s="4" t="n"/>
+      <c r="G91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -3025,8 +3047,7 @@
         <v/>
       </c>
       <c r="F92" s="4" t="n"/>
-      <c r="G92" s="3" t="n"/>
-      <c r="H92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
@@ -3042,8 +3063,7 @@
         <v/>
       </c>
       <c r="F93" s="4" t="n"/>
-      <c r="G93" s="3" t="n"/>
-      <c r="H93" s="4" t="n"/>
+      <c r="G93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -3059,8 +3079,7 @@
         <v/>
       </c>
       <c r="F94" s="4" t="n"/>
-      <c r="G94" s="3" t="n"/>
-      <c r="H94" s="4" t="n"/>
+      <c r="G94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n"/>
@@ -3069,8 +3088,7 @@
       <c r="D95" s="4" t="n"/>
       <c r="E95" s="4" t="n"/>
       <c r="F95" s="4" t="n"/>
-      <c r="G95" s="3" t="n"/>
-      <c r="H95" s="4" t="n"/>
+      <c r="G95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -3086,8 +3104,7 @@
         <v/>
       </c>
       <c r="F96" s="4" t="n"/>
-      <c r="G96" s="3" t="n"/>
-      <c r="H96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
@@ -3103,8 +3120,7 @@
         <v/>
       </c>
       <c r="F97" s="4" t="n"/>
-      <c r="G97" s="3" t="n"/>
-      <c r="H97" s="4" t="n"/>
+      <c r="G97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -3113,8 +3129,7 @@
       <c r="D98" s="4" t="n"/>
       <c r="E98" s="4" t="n"/>
       <c r="F98" s="4" t="n"/>
-      <c r="G98" s="3" t="n"/>
-      <c r="H98" s="4" t="n"/>
+      <c r="G98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
@@ -3130,8 +3145,7 @@
         <v/>
       </c>
       <c r="F99" s="4" t="n"/>
-      <c r="G99" s="3" t="n"/>
-      <c r="H99" s="4" t="n"/>
+      <c r="G99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -3147,8 +3161,7 @@
         <v/>
       </c>
       <c r="F100" s="4" t="n"/>
-      <c r="G100" s="3" t="n"/>
-      <c r="H100" s="4" t="n"/>
+      <c r="G100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n"/>
@@ -3157,8 +3170,7 @@
       <c r="D101" s="4" t="n"/>
       <c r="E101" s="4" t="n"/>
       <c r="F101" s="4" t="n"/>
-      <c r="G101" s="3" t="n"/>
-      <c r="H101" s="4" t="n"/>
+      <c r="G101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
@@ -3171,8 +3183,2132 @@
       <c r="D102" s="4" t="n"/>
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="n"/>
-      <c r="G102" s="3" t="n"/>
-      <c r="H102" s="4" t="n"/>
+      <c r="G102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Status: identifiziert → bestellt → geliefert → verbaut (Auswahl in Spalte H)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H22 H23 H26 H27 H28 H29 H30 H31 H32 H35 H36 H37 H38 H39 H40 H41 H42 H43 H46 H47 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"identifiziert,bestellt,geliefert,verbaut"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F106"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Bestellliste nach Hersteller / Shop (Mengen für Vollausbau, 4 Proben)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Teil</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Menge Vollausbau</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Einzelpreis inkl. MwSt. (€)</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Gesamt inkl. MwSt. (€)</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f>Bestellliste!A18</f>
+        <v/>
+      </c>
+      <c r="B6">
+        <f>IF(Bestellliste!C18="","",IF(Bestellliste!F18="x",4*Bestellliste!C18,Bestellliste!C18))</f>
+        <v/>
+      </c>
+      <c r="C6" s="15">
+        <f>IF(Bestellliste!D18="","",Bestellliste!D18)</f>
+        <v/>
+      </c>
+      <c r="D6" s="15">
+        <f>IF(AND(ISNUMBER(B6),ISNUMBER(C6)),B6*C6,0)</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>IF(Bestellliste!G18="","",Bestellliste!G18)</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>IF(Bestellliste!H18="","",Bestellliste!H18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <f>Bestellliste!A23</f>
+        <v/>
+      </c>
+      <c r="B7">
+        <f>IF(Bestellliste!C23="","",IF(Bestellliste!F23="x",4*Bestellliste!C23,Bestellliste!C23))</f>
+        <v/>
+      </c>
+      <c r="C7" s="15">
+        <f>IF(Bestellliste!D23="","",Bestellliste!D23)</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>IF(AND(ISNUMBER(B7),ISNUMBER(C7)),B7*C7,0)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>IF(Bestellliste!G23="","",Bestellliste!G23)</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>IF(Bestellliste!H23="","",Bestellliste!H23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>Bestellliste!A32</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IF(Bestellliste!C32="","",IF(Bestellliste!F32="x",4*Bestellliste!C32,Bestellliste!C32))</f>
+        <v/>
+      </c>
+      <c r="C8" s="15">
+        <f>IF(Bestellliste!D32="","",Bestellliste!D32)</f>
+        <v/>
+      </c>
+      <c r="D8" s="15">
+        <f>IF(AND(ISNUMBER(B8),ISNUMBER(C8)),B8*C8,0)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IF(Bestellliste!G32="","",Bestellliste!G32)</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IF(Bestellliste!H32="","",Bestellliste!H32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>Bestellliste!A42</f>
+        <v/>
+      </c>
+      <c r="B9">
+        <f>IF(Bestellliste!C42="","",IF(Bestellliste!F42="x",4*Bestellliste!C42,Bestellliste!C42))</f>
+        <v/>
+      </c>
+      <c r="C9" s="15">
+        <f>IF(Bestellliste!D42="","",Bestellliste!D42)</f>
+        <v/>
+      </c>
+      <c r="D9" s="15">
+        <f>IF(AND(ISNUMBER(B9),ISNUMBER(C9)),B9*C9,0)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>IF(Bestellliste!G42="","",Bestellliste!G42)</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>IF(Bestellliste!H42="","",Bestellliste!H42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <f>Bestellliste!A60</f>
+        <v/>
+      </c>
+      <c r="B10">
+        <f>IF(Bestellliste!C60="","",IF(Bestellliste!F60="x",4*Bestellliste!C60,Bestellliste!C60))</f>
+        <v/>
+      </c>
+      <c r="C10" s="15">
+        <f>IF(Bestellliste!D60="","",Bestellliste!D60)</f>
+        <v/>
+      </c>
+      <c r="D10" s="15">
+        <f>IF(AND(ISNUMBER(B10),ISNUMBER(C10)),B10*C10,0)</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>IF(Bestellliste!G60="","",Bestellliste!G60)</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>IF(Bestellliste!H60="","",Bestellliste!H60)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Summe Amazon</t>
+        </is>
+      </c>
+      <c r="D11" s="15">
+        <f>SUM(D6:D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>DOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>Bestellliste!A6</f>
+        <v/>
+      </c>
+      <c r="B14">
+        <f>IF(Bestellliste!C6="","",IF(Bestellliste!F6="x",4*Bestellliste!C6,Bestellliste!C6))</f>
+        <v/>
+      </c>
+      <c r="C14" s="15">
+        <f>IF(Bestellliste!D6="","",Bestellliste!D6)</f>
+        <v/>
+      </c>
+      <c r="D14" s="15">
+        <f>IF(AND(ISNUMBER(B14),ISNUMBER(C14)),B14*C14,0)</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>IF(Bestellliste!G6="","",Bestellliste!G6)</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>IF(Bestellliste!H6="","",Bestellliste!H6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <f>Bestellliste!A7</f>
+        <v/>
+      </c>
+      <c r="B15">
+        <f>IF(Bestellliste!C7="","",IF(Bestellliste!F7="x",4*Bestellliste!C7,Bestellliste!C7))</f>
+        <v/>
+      </c>
+      <c r="C15" s="15">
+        <f>IF(Bestellliste!D7="","",Bestellliste!D7)</f>
+        <v/>
+      </c>
+      <c r="D15" s="15">
+        <f>IF(AND(ISNUMBER(B15),ISNUMBER(C15)),B15*C15,0)</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>IF(Bestellliste!G7="","",Bestellliste!G7)</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>IF(Bestellliste!H7="","",Bestellliste!H7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <f>Bestellliste!A8</f>
+        <v/>
+      </c>
+      <c r="B16">
+        <f>IF(Bestellliste!C8="","",IF(Bestellliste!F8="x",4*Bestellliste!C8,Bestellliste!C8))</f>
+        <v/>
+      </c>
+      <c r="C16" s="15">
+        <f>IF(Bestellliste!D8="","",Bestellliste!D8)</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>IF(AND(ISNUMBER(B16),ISNUMBER(C16)),B16*C16,0)</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>IF(Bestellliste!G8="","",Bestellliste!G8)</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>IF(Bestellliste!H8="","",Bestellliste!H8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <f>Bestellliste!A9</f>
+        <v/>
+      </c>
+      <c r="B17">
+        <f>IF(Bestellliste!C9="","",IF(Bestellliste!F9="x",4*Bestellliste!C9,Bestellliste!C9))</f>
+        <v/>
+      </c>
+      <c r="C17" s="15">
+        <f>IF(Bestellliste!D9="","",Bestellliste!D9)</f>
+        <v/>
+      </c>
+      <c r="D17" s="15">
+        <f>IF(AND(ISNUMBER(B17),ISNUMBER(C17)),B17*C17,0)</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>IF(Bestellliste!G9="","",Bestellliste!G9)</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>IF(Bestellliste!H9="","",Bestellliste!H9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <f>Bestellliste!A10</f>
+        <v/>
+      </c>
+      <c r="B18">
+        <f>IF(Bestellliste!C10="","",IF(Bestellliste!F10="x",4*Bestellliste!C10,Bestellliste!C10))</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>IF(Bestellliste!D10="","",Bestellliste!D10)</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>IF(AND(ISNUMBER(B18),ISNUMBER(C18)),B18*C18,0)</f>
+        <v/>
+      </c>
+      <c r="E18">
+        <f>IF(Bestellliste!G10="","",Bestellliste!G10)</f>
+        <v/>
+      </c>
+      <c r="F18">
+        <f>IF(Bestellliste!H10="","",Bestellliste!H10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <f>Bestellliste!A11</f>
+        <v/>
+      </c>
+      <c r="B19">
+        <f>IF(Bestellliste!C11="","",IF(Bestellliste!F11="x",4*Bestellliste!C11,Bestellliste!C11))</f>
+        <v/>
+      </c>
+      <c r="C19" s="15">
+        <f>IF(Bestellliste!D11="","",Bestellliste!D11)</f>
+        <v/>
+      </c>
+      <c r="D19" s="15">
+        <f>IF(AND(ISNUMBER(B19),ISNUMBER(C19)),B19*C19,0)</f>
+        <v/>
+      </c>
+      <c r="E19">
+        <f>IF(Bestellliste!G11="","",Bestellliste!G11)</f>
+        <v/>
+      </c>
+      <c r="F19">
+        <f>IF(Bestellliste!H11="","",Bestellliste!H11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <f>Bestellliste!A12</f>
+        <v/>
+      </c>
+      <c r="B20">
+        <f>IF(Bestellliste!C12="","",IF(Bestellliste!F12="x",4*Bestellliste!C12,Bestellliste!C12))</f>
+        <v/>
+      </c>
+      <c r="C20" s="15">
+        <f>IF(Bestellliste!D12="","",Bestellliste!D12)</f>
+        <v/>
+      </c>
+      <c r="D20" s="15">
+        <f>IF(AND(ISNUMBER(B20),ISNUMBER(C20)),B20*C20,0)</f>
+        <v/>
+      </c>
+      <c r="E20">
+        <f>IF(Bestellliste!G12="","",Bestellliste!G12)</f>
+        <v/>
+      </c>
+      <c r="F20">
+        <f>IF(Bestellliste!H12="","",Bestellliste!H12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <f>Bestellliste!A13</f>
+        <v/>
+      </c>
+      <c r="B21">
+        <f>IF(Bestellliste!C13="","",IF(Bestellliste!F13="x",4*Bestellliste!C13,Bestellliste!C13))</f>
+        <v/>
+      </c>
+      <c r="C21" s="15">
+        <f>IF(Bestellliste!D13="","",Bestellliste!D13)</f>
+        <v/>
+      </c>
+      <c r="D21" s="15">
+        <f>IF(AND(ISNUMBER(B21),ISNUMBER(C21)),B21*C21,0)</f>
+        <v/>
+      </c>
+      <c r="E21">
+        <f>IF(Bestellliste!G13="","",Bestellliste!G13)</f>
+        <v/>
+      </c>
+      <c r="F21">
+        <f>IF(Bestellliste!H13="","",Bestellliste!H13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <f>Bestellliste!A14</f>
+        <v/>
+      </c>
+      <c r="B22">
+        <f>IF(Bestellliste!C14="","",IF(Bestellliste!F14="x",4*Bestellliste!C14,Bestellliste!C14))</f>
+        <v/>
+      </c>
+      <c r="C22" s="15">
+        <f>IF(Bestellliste!D14="","",Bestellliste!D14)</f>
+        <v/>
+      </c>
+      <c r="D22" s="15">
+        <f>IF(AND(ISNUMBER(B22),ISNUMBER(C22)),B22*C22,0)</f>
+        <v/>
+      </c>
+      <c r="E22">
+        <f>IF(Bestellliste!G14="","",Bestellliste!G14)</f>
+        <v/>
+      </c>
+      <c r="F22">
+        <f>IF(Bestellliste!H14="","",Bestellliste!H14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <f>Bestellliste!A17</f>
+        <v/>
+      </c>
+      <c r="B23">
+        <f>IF(Bestellliste!C17="","",IF(Bestellliste!F17="x",4*Bestellliste!C17,Bestellliste!C17))</f>
+        <v/>
+      </c>
+      <c r="C23" s="15">
+        <f>IF(Bestellliste!D17="","",Bestellliste!D17)</f>
+        <v/>
+      </c>
+      <c r="D23" s="15">
+        <f>IF(AND(ISNUMBER(B23),ISNUMBER(C23)),B23*C23,0)</f>
+        <v/>
+      </c>
+      <c r="E23">
+        <f>IF(Bestellliste!G17="","",Bestellliste!G17)</f>
+        <v/>
+      </c>
+      <c r="F23">
+        <f>IF(Bestellliste!H17="","",Bestellliste!H17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <f>Bestellliste!A19</f>
+        <v/>
+      </c>
+      <c r="B24">
+        <f>IF(Bestellliste!C19="","",IF(Bestellliste!F19="x",4*Bestellliste!C19,Bestellliste!C19))</f>
+        <v/>
+      </c>
+      <c r="C24" s="15">
+        <f>IF(Bestellliste!D19="","",Bestellliste!D19)</f>
+        <v/>
+      </c>
+      <c r="D24" s="15">
+        <f>IF(AND(ISNUMBER(B24),ISNUMBER(C24)),B24*C24,0)</f>
+        <v/>
+      </c>
+      <c r="E24">
+        <f>IF(Bestellliste!G19="","",Bestellliste!G19)</f>
+        <v/>
+      </c>
+      <c r="F24">
+        <f>IF(Bestellliste!H19="","",Bestellliste!H19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <f>Bestellliste!A27</f>
+        <v/>
+      </c>
+      <c r="B25">
+        <f>IF(Bestellliste!C27="","",IF(Bestellliste!F27="x",4*Bestellliste!C27,Bestellliste!C27))</f>
+        <v/>
+      </c>
+      <c r="C25" s="15">
+        <f>IF(Bestellliste!D27="","",Bestellliste!D27)</f>
+        <v/>
+      </c>
+      <c r="D25" s="15">
+        <f>IF(AND(ISNUMBER(B25),ISNUMBER(C25)),B25*C25,0)</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>IF(Bestellliste!G27="","",Bestellliste!G27)</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>IF(Bestellliste!H27="","",Bestellliste!H27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <f>Bestellliste!A30</f>
+        <v/>
+      </c>
+      <c r="B26">
+        <f>IF(Bestellliste!C30="","",IF(Bestellliste!F30="x",4*Bestellliste!C30,Bestellliste!C30))</f>
+        <v/>
+      </c>
+      <c r="C26" s="15">
+        <f>IF(Bestellliste!D30="","",Bestellliste!D30)</f>
+        <v/>
+      </c>
+      <c r="D26" s="15">
+        <f>IF(AND(ISNUMBER(B26),ISNUMBER(C26)),B26*C26,0)</f>
+        <v/>
+      </c>
+      <c r="E26">
+        <f>IF(Bestellliste!G30="","",Bestellliste!G30)</f>
+        <v/>
+      </c>
+      <c r="F26">
+        <f>IF(Bestellliste!H30="","",Bestellliste!H30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <f>Bestellliste!A31</f>
+        <v/>
+      </c>
+      <c r="B27">
+        <f>IF(Bestellliste!C31="","",IF(Bestellliste!F31="x",4*Bestellliste!C31,Bestellliste!C31))</f>
+        <v/>
+      </c>
+      <c r="C27" s="15">
+        <f>IF(Bestellliste!D31="","",Bestellliste!D31)</f>
+        <v/>
+      </c>
+      <c r="D27" s="15">
+        <f>IF(AND(ISNUMBER(B27),ISNUMBER(C27)),B27*C27,0)</f>
+        <v/>
+      </c>
+      <c r="E27">
+        <f>IF(Bestellliste!G31="","",Bestellliste!G31)</f>
+        <v/>
+      </c>
+      <c r="F27">
+        <f>IF(Bestellliste!H31="","",Bestellliste!H31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <f>Bestellliste!A35</f>
+        <v/>
+      </c>
+      <c r="B28">
+        <f>IF(Bestellliste!C35="","",IF(Bestellliste!F35="x",4*Bestellliste!C35,Bestellliste!C35))</f>
+        <v/>
+      </c>
+      <c r="C28" s="15">
+        <f>IF(Bestellliste!D35="","",Bestellliste!D35)</f>
+        <v/>
+      </c>
+      <c r="D28" s="15">
+        <f>IF(AND(ISNUMBER(B28),ISNUMBER(C28)),B28*C28,0)</f>
+        <v/>
+      </c>
+      <c r="E28">
+        <f>IF(Bestellliste!G35="","",Bestellliste!G35)</f>
+        <v/>
+      </c>
+      <c r="F28">
+        <f>IF(Bestellliste!H35="","",Bestellliste!H35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <f>Bestellliste!A36</f>
+        <v/>
+      </c>
+      <c r="B29">
+        <f>IF(Bestellliste!C36="","",IF(Bestellliste!F36="x",4*Bestellliste!C36,Bestellliste!C36))</f>
+        <v/>
+      </c>
+      <c r="C29" s="15">
+        <f>IF(Bestellliste!D36="","",Bestellliste!D36)</f>
+        <v/>
+      </c>
+      <c r="D29" s="15">
+        <f>IF(AND(ISNUMBER(B29),ISNUMBER(C29)),B29*C29,0)</f>
+        <v/>
+      </c>
+      <c r="E29">
+        <f>IF(Bestellliste!G36="","",Bestellliste!G36)</f>
+        <v/>
+      </c>
+      <c r="F29">
+        <f>IF(Bestellliste!H36="","",Bestellliste!H36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <f>Bestellliste!A38</f>
+        <v/>
+      </c>
+      <c r="B30">
+        <f>IF(Bestellliste!C38="","",IF(Bestellliste!F38="x",4*Bestellliste!C38,Bestellliste!C38))</f>
+        <v/>
+      </c>
+      <c r="C30" s="15">
+        <f>IF(Bestellliste!D38="","",Bestellliste!D38)</f>
+        <v/>
+      </c>
+      <c r="D30" s="15">
+        <f>IF(AND(ISNUMBER(B30),ISNUMBER(C30)),B30*C30,0)</f>
+        <v/>
+      </c>
+      <c r="E30">
+        <f>IF(Bestellliste!G38="","",Bestellliste!G38)</f>
+        <v/>
+      </c>
+      <c r="F30">
+        <f>IF(Bestellliste!H38="","",Bestellliste!H38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <f>Bestellliste!A39</f>
+        <v/>
+      </c>
+      <c r="B31">
+        <f>IF(Bestellliste!C39="","",IF(Bestellliste!F39="x",4*Bestellliste!C39,Bestellliste!C39))</f>
+        <v/>
+      </c>
+      <c r="C31" s="15">
+        <f>IF(Bestellliste!D39="","",Bestellliste!D39)</f>
+        <v/>
+      </c>
+      <c r="D31" s="15">
+        <f>IF(AND(ISNUMBER(B31),ISNUMBER(C31)),B31*C31,0)</f>
+        <v/>
+      </c>
+      <c r="E31">
+        <f>IF(Bestellliste!G39="","",Bestellliste!G39)</f>
+        <v/>
+      </c>
+      <c r="F31">
+        <f>IF(Bestellliste!H39="","",Bestellliste!H39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <f>Bestellliste!A40</f>
+        <v/>
+      </c>
+      <c r="B32">
+        <f>IF(Bestellliste!C40="","",IF(Bestellliste!F40="x",4*Bestellliste!C40,Bestellliste!C40))</f>
+        <v/>
+      </c>
+      <c r="C32" s="15">
+        <f>IF(Bestellliste!D40="","",Bestellliste!D40)</f>
+        <v/>
+      </c>
+      <c r="D32" s="15">
+        <f>IF(AND(ISNUMBER(B32),ISNUMBER(C32)),B32*C32,0)</f>
+        <v/>
+      </c>
+      <c r="E32">
+        <f>IF(Bestellliste!G40="","",Bestellliste!G40)</f>
+        <v/>
+      </c>
+      <c r="F32">
+        <f>IF(Bestellliste!H40="","",Bestellliste!H40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <f>Bestellliste!A46</f>
+        <v/>
+      </c>
+      <c r="B33">
+        <f>IF(Bestellliste!C46="","",IF(Bestellliste!F46="x",4*Bestellliste!C46,Bestellliste!C46))</f>
+        <v/>
+      </c>
+      <c r="C33" s="15">
+        <f>IF(Bestellliste!D46="","",Bestellliste!D46)</f>
+        <v/>
+      </c>
+      <c r="D33" s="15">
+        <f>IF(AND(ISNUMBER(B33),ISNUMBER(C33)),B33*C33,0)</f>
+        <v/>
+      </c>
+      <c r="E33">
+        <f>IF(Bestellliste!G46="","",Bestellliste!G46)</f>
+        <v/>
+      </c>
+      <c r="F33">
+        <f>IF(Bestellliste!H46="","",Bestellliste!H46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <f>Bestellliste!A52</f>
+        <v/>
+      </c>
+      <c r="B34">
+        <f>IF(Bestellliste!C52="","",IF(Bestellliste!F52="x",4*Bestellliste!C52,Bestellliste!C52))</f>
+        <v/>
+      </c>
+      <c r="C34" s="15">
+        <f>IF(Bestellliste!D52="","",Bestellliste!D52)</f>
+        <v/>
+      </c>
+      <c r="D34" s="15">
+        <f>IF(AND(ISNUMBER(B34),ISNUMBER(C34)),B34*C34,0)</f>
+        <v/>
+      </c>
+      <c r="E34">
+        <f>IF(Bestellliste!G52="","",Bestellliste!G52)</f>
+        <v/>
+      </c>
+      <c r="F34">
+        <f>IF(Bestellliste!H52="","",Bestellliste!H52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <f>Bestellliste!A63</f>
+        <v/>
+      </c>
+      <c r="B35">
+        <f>IF(Bestellliste!C63="","",IF(Bestellliste!F63="x",4*Bestellliste!C63,Bestellliste!C63))</f>
+        <v/>
+      </c>
+      <c r="C35" s="15">
+        <f>IF(Bestellliste!D63="","",Bestellliste!D63)</f>
+        <v/>
+      </c>
+      <c r="D35" s="15">
+        <f>IF(AND(ISNUMBER(B35),ISNUMBER(C35)),B35*C35,0)</f>
+        <v/>
+      </c>
+      <c r="E35">
+        <f>IF(Bestellliste!G63="","",Bestellliste!G63)</f>
+        <v/>
+      </c>
+      <c r="F35">
+        <f>IF(Bestellliste!H63="","",Bestellliste!H63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <f>Bestellliste!A64</f>
+        <v/>
+      </c>
+      <c r="B36">
+        <f>IF(Bestellliste!C64="","",IF(Bestellliste!F64="x",4*Bestellliste!C64,Bestellliste!C64))</f>
+        <v/>
+      </c>
+      <c r="C36" s="15">
+        <f>IF(Bestellliste!D64="","",Bestellliste!D64)</f>
+        <v/>
+      </c>
+      <c r="D36" s="15">
+        <f>IF(AND(ISNUMBER(B36),ISNUMBER(C36)),B36*C36,0)</f>
+        <v/>
+      </c>
+      <c r="E36">
+        <f>IF(Bestellliste!G64="","",Bestellliste!G64)</f>
+        <v/>
+      </c>
+      <c r="F36">
+        <f>IF(Bestellliste!H64="","",Bestellliste!H64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <f>Bestellliste!A65</f>
+        <v/>
+      </c>
+      <c r="B37">
+        <f>IF(Bestellliste!C65="","",IF(Bestellliste!F65="x",4*Bestellliste!C65,Bestellliste!C65))</f>
+        <v/>
+      </c>
+      <c r="C37" s="15">
+        <f>IF(Bestellliste!D65="","",Bestellliste!D65)</f>
+        <v/>
+      </c>
+      <c r="D37" s="15">
+        <f>IF(AND(ISNUMBER(B37),ISNUMBER(C37)),B37*C37,0)</f>
+        <v/>
+      </c>
+      <c r="E37">
+        <f>IF(Bestellliste!G65="","",Bestellliste!G65)</f>
+        <v/>
+      </c>
+      <c r="F37">
+        <f>IF(Bestellliste!H65="","",Bestellliste!H65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <f>Bestellliste!A66</f>
+        <v/>
+      </c>
+      <c r="B38">
+        <f>IF(Bestellliste!C66="","",IF(Bestellliste!F66="x",4*Bestellliste!C66,Bestellliste!C66))</f>
+        <v/>
+      </c>
+      <c r="C38" s="15">
+        <f>IF(Bestellliste!D66="","",Bestellliste!D66)</f>
+        <v/>
+      </c>
+      <c r="D38" s="15">
+        <f>IF(AND(ISNUMBER(B38),ISNUMBER(C38)),B38*C38,0)</f>
+        <v/>
+      </c>
+      <c r="E38">
+        <f>IF(Bestellliste!G66="","",Bestellliste!G66)</f>
+        <v/>
+      </c>
+      <c r="F38">
+        <f>IF(Bestellliste!H66="","",Bestellliste!H66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <f>Bestellliste!A67</f>
+        <v/>
+      </c>
+      <c r="B39">
+        <f>IF(Bestellliste!C67="","",IF(Bestellliste!F67="x",4*Bestellliste!C67,Bestellliste!C67))</f>
+        <v/>
+      </c>
+      <c r="C39" s="15">
+        <f>IF(Bestellliste!D67="","",Bestellliste!D67)</f>
+        <v/>
+      </c>
+      <c r="D39" s="15">
+        <f>IF(AND(ISNUMBER(B39),ISNUMBER(C39)),B39*C39,0)</f>
+        <v/>
+      </c>
+      <c r="E39">
+        <f>IF(Bestellliste!G67="","",Bestellliste!G67)</f>
+        <v/>
+      </c>
+      <c r="F39">
+        <f>IF(Bestellliste!H67="","",Bestellliste!H67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <f>Bestellliste!A68</f>
+        <v/>
+      </c>
+      <c r="B40">
+        <f>IF(Bestellliste!C68="","",IF(Bestellliste!F68="x",4*Bestellliste!C68,Bestellliste!C68))</f>
+        <v/>
+      </c>
+      <c r="C40" s="15">
+        <f>IF(Bestellliste!D68="","",Bestellliste!D68)</f>
+        <v/>
+      </c>
+      <c r="D40" s="15">
+        <f>IF(AND(ISNUMBER(B40),ISNUMBER(C40)),B40*C40,0)</f>
+        <v/>
+      </c>
+      <c r="E40">
+        <f>IF(Bestellliste!G68="","",Bestellliste!G68)</f>
+        <v/>
+      </c>
+      <c r="F40">
+        <f>IF(Bestellliste!H68="","",Bestellliste!H68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <f>Bestellliste!A69</f>
+        <v/>
+      </c>
+      <c r="B41">
+        <f>IF(Bestellliste!C69="","",IF(Bestellliste!F69="x",4*Bestellliste!C69,Bestellliste!C69))</f>
+        <v/>
+      </c>
+      <c r="C41" s="15">
+        <f>IF(Bestellliste!D69="","",Bestellliste!D69)</f>
+        <v/>
+      </c>
+      <c r="D41" s="15">
+        <f>IF(AND(ISNUMBER(B41),ISNUMBER(C41)),B41*C41,0)</f>
+        <v/>
+      </c>
+      <c r="E41">
+        <f>IF(Bestellliste!G69="","",Bestellliste!G69)</f>
+        <v/>
+      </c>
+      <c r="F41">
+        <f>IF(Bestellliste!H69="","",Bestellliste!H69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <f>Bestellliste!A70</f>
+        <v/>
+      </c>
+      <c r="B42">
+        <f>IF(Bestellliste!C70="","",IF(Bestellliste!F70="x",4*Bestellliste!C70,Bestellliste!C70))</f>
+        <v/>
+      </c>
+      <c r="C42" s="15">
+        <f>IF(Bestellliste!D70="","",Bestellliste!D70)</f>
+        <v/>
+      </c>
+      <c r="D42" s="15">
+        <f>IF(AND(ISNUMBER(B42),ISNUMBER(C42)),B42*C42,0)</f>
+        <v/>
+      </c>
+      <c r="E42">
+        <f>IF(Bestellliste!G70="","",Bestellliste!G70)</f>
+        <v/>
+      </c>
+      <c r="F42">
+        <f>IF(Bestellliste!H70="","",Bestellliste!H70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <f>Bestellliste!A71</f>
+        <v/>
+      </c>
+      <c r="B43">
+        <f>IF(Bestellliste!C71="","",IF(Bestellliste!F71="x",4*Bestellliste!C71,Bestellliste!C71))</f>
+        <v/>
+      </c>
+      <c r="C43" s="15">
+        <f>IF(Bestellliste!D71="","",Bestellliste!D71)</f>
+        <v/>
+      </c>
+      <c r="D43" s="15">
+        <f>IF(AND(ISNUMBER(B43),ISNUMBER(C43)),B43*C43,0)</f>
+        <v/>
+      </c>
+      <c r="E43">
+        <f>IF(Bestellliste!G71="","",Bestellliste!G71)</f>
+        <v/>
+      </c>
+      <c r="F43">
+        <f>IF(Bestellliste!H71="","",Bestellliste!H71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <f>Bestellliste!A72</f>
+        <v/>
+      </c>
+      <c r="B44">
+        <f>IF(Bestellliste!C72="","",IF(Bestellliste!F72="x",4*Bestellliste!C72,Bestellliste!C72))</f>
+        <v/>
+      </c>
+      <c r="C44" s="15">
+        <f>IF(Bestellliste!D72="","",Bestellliste!D72)</f>
+        <v/>
+      </c>
+      <c r="D44" s="15">
+        <f>IF(AND(ISNUMBER(B44),ISNUMBER(C44)),B44*C44,0)</f>
+        <v/>
+      </c>
+      <c r="E44">
+        <f>IF(Bestellliste!G72="","",Bestellliste!G72)</f>
+        <v/>
+      </c>
+      <c r="F44">
+        <f>IF(Bestellliste!H72="","",Bestellliste!H72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <f>Bestellliste!A73</f>
+        <v/>
+      </c>
+      <c r="B45">
+        <f>IF(Bestellliste!C73="","",IF(Bestellliste!F73="x",4*Bestellliste!C73,Bestellliste!C73))</f>
+        <v/>
+      </c>
+      <c r="C45" s="15">
+        <f>IF(Bestellliste!D73="","",Bestellliste!D73)</f>
+        <v/>
+      </c>
+      <c r="D45" s="15">
+        <f>IF(AND(ISNUMBER(B45),ISNUMBER(C45)),B45*C45,0)</f>
+        <v/>
+      </c>
+      <c r="E45">
+        <f>IF(Bestellliste!G73="","",Bestellliste!G73)</f>
+        <v/>
+      </c>
+      <c r="F45">
+        <f>IF(Bestellliste!H73="","",Bestellliste!H73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <f>Bestellliste!A74</f>
+        <v/>
+      </c>
+      <c r="B46">
+        <f>IF(Bestellliste!C74="","",IF(Bestellliste!F74="x",4*Bestellliste!C74,Bestellliste!C74))</f>
+        <v/>
+      </c>
+      <c r="C46" s="15">
+        <f>IF(Bestellliste!D74="","",Bestellliste!D74)</f>
+        <v/>
+      </c>
+      <c r="D46" s="15">
+        <f>IF(AND(ISNUMBER(B46),ISNUMBER(C46)),B46*C46,0)</f>
+        <v/>
+      </c>
+      <c r="E46">
+        <f>IF(Bestellliste!G74="","",Bestellliste!G74)</f>
+        <v/>
+      </c>
+      <c r="F46">
+        <f>IF(Bestellliste!H74="","",Bestellliste!H74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <f>Bestellliste!A75</f>
+        <v/>
+      </c>
+      <c r="B47">
+        <f>IF(Bestellliste!C75="","",IF(Bestellliste!F75="x",4*Bestellliste!C75,Bestellliste!C75))</f>
+        <v/>
+      </c>
+      <c r="C47" s="15">
+        <f>IF(Bestellliste!D75="","",Bestellliste!D75)</f>
+        <v/>
+      </c>
+      <c r="D47" s="15">
+        <f>IF(AND(ISNUMBER(B47),ISNUMBER(C47)),B47*C47,0)</f>
+        <v/>
+      </c>
+      <c r="E47">
+        <f>IF(Bestellliste!G75="","",Bestellliste!G75)</f>
+        <v/>
+      </c>
+      <c r="F47">
+        <f>IF(Bestellliste!H75="","",Bestellliste!H75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <f>Bestellliste!A76</f>
+        <v/>
+      </c>
+      <c r="B48">
+        <f>IF(Bestellliste!C76="","",IF(Bestellliste!F76="x",4*Bestellliste!C76,Bestellliste!C76))</f>
+        <v/>
+      </c>
+      <c r="C48" s="15">
+        <f>IF(Bestellliste!D76="","",Bestellliste!D76)</f>
+        <v/>
+      </c>
+      <c r="D48" s="15">
+        <f>IF(AND(ISNUMBER(B48),ISNUMBER(C48)),B48*C48,0)</f>
+        <v/>
+      </c>
+      <c r="E48">
+        <f>IF(Bestellliste!G76="","",Bestellliste!G76)</f>
+        <v/>
+      </c>
+      <c r="F48">
+        <f>IF(Bestellliste!H76="","",Bestellliste!H76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <f>Bestellliste!A77</f>
+        <v/>
+      </c>
+      <c r="B49">
+        <f>IF(Bestellliste!C77="","",IF(Bestellliste!F77="x",4*Bestellliste!C77,Bestellliste!C77))</f>
+        <v/>
+      </c>
+      <c r="C49" s="15">
+        <f>IF(Bestellliste!D77="","",Bestellliste!D77)</f>
+        <v/>
+      </c>
+      <c r="D49" s="15">
+        <f>IF(AND(ISNUMBER(B49),ISNUMBER(C49)),B49*C49,0)</f>
+        <v/>
+      </c>
+      <c r="E49">
+        <f>IF(Bestellliste!G77="","",Bestellliste!G77)</f>
+        <v/>
+      </c>
+      <c r="F49">
+        <f>IF(Bestellliste!H77="","",Bestellliste!H77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <f>Bestellliste!A78</f>
+        <v/>
+      </c>
+      <c r="B50">
+        <f>IF(Bestellliste!C78="","",IF(Bestellliste!F78="x",4*Bestellliste!C78,Bestellliste!C78))</f>
+        <v/>
+      </c>
+      <c r="C50" s="15">
+        <f>IF(Bestellliste!D78="","",Bestellliste!D78)</f>
+        <v/>
+      </c>
+      <c r="D50" s="15">
+        <f>IF(AND(ISNUMBER(B50),ISNUMBER(C50)),B50*C50,0)</f>
+        <v/>
+      </c>
+      <c r="E50">
+        <f>IF(Bestellliste!G78="","",Bestellliste!G78)</f>
+        <v/>
+      </c>
+      <c r="F50">
+        <f>IF(Bestellliste!H78="","",Bestellliste!H78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <f>Bestellliste!A79</f>
+        <v/>
+      </c>
+      <c r="B51">
+        <f>IF(Bestellliste!C79="","",IF(Bestellliste!F79="x",4*Bestellliste!C79,Bestellliste!C79))</f>
+        <v/>
+      </c>
+      <c r="C51" s="15">
+        <f>IF(Bestellliste!D79="","",Bestellliste!D79)</f>
+        <v/>
+      </c>
+      <c r="D51" s="15">
+        <f>IF(AND(ISNUMBER(B51),ISNUMBER(C51)),B51*C51,0)</f>
+        <v/>
+      </c>
+      <c r="E51">
+        <f>IF(Bestellliste!G79="","",Bestellliste!G79)</f>
+        <v/>
+      </c>
+      <c r="F51">
+        <f>IF(Bestellliste!H79="","",Bestellliste!H79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <f>Bestellliste!A80</f>
+        <v/>
+      </c>
+      <c r="B52">
+        <f>IF(Bestellliste!C80="","",IF(Bestellliste!F80="x",4*Bestellliste!C80,Bestellliste!C80))</f>
+        <v/>
+      </c>
+      <c r="C52" s="15">
+        <f>IF(Bestellliste!D80="","",Bestellliste!D80)</f>
+        <v/>
+      </c>
+      <c r="D52" s="15">
+        <f>IF(AND(ISNUMBER(B52),ISNUMBER(C52)),B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="E52">
+        <f>IF(Bestellliste!G80="","",Bestellliste!G80)</f>
+        <v/>
+      </c>
+      <c r="F52">
+        <f>IF(Bestellliste!H80="","",Bestellliste!H80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <f>Bestellliste!A81</f>
+        <v/>
+      </c>
+      <c r="B53">
+        <f>IF(Bestellliste!C81="","",IF(Bestellliste!F81="x",4*Bestellliste!C81,Bestellliste!C81))</f>
+        <v/>
+      </c>
+      <c r="C53" s="15">
+        <f>IF(Bestellliste!D81="","",Bestellliste!D81)</f>
+        <v/>
+      </c>
+      <c r="D53" s="15">
+        <f>IF(AND(ISNUMBER(B53),ISNUMBER(C53)),B53*C53,0)</f>
+        <v/>
+      </c>
+      <c r="E53">
+        <f>IF(Bestellliste!G81="","",Bestellliste!G81)</f>
+        <v/>
+      </c>
+      <c r="F53">
+        <f>IF(Bestellliste!H81="","",Bestellliste!H81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <f>Bestellliste!A82</f>
+        <v/>
+      </c>
+      <c r="B54">
+        <f>IF(Bestellliste!C82="","",IF(Bestellliste!F82="x",4*Bestellliste!C82,Bestellliste!C82))</f>
+        <v/>
+      </c>
+      <c r="C54" s="15">
+        <f>IF(Bestellliste!D82="","",Bestellliste!D82)</f>
+        <v/>
+      </c>
+      <c r="D54" s="15">
+        <f>IF(AND(ISNUMBER(B54),ISNUMBER(C54)),B54*C54,0)</f>
+        <v/>
+      </c>
+      <c r="E54">
+        <f>IF(Bestellliste!G82="","",Bestellliste!G82)</f>
+        <v/>
+      </c>
+      <c r="F54">
+        <f>IF(Bestellliste!H82="","",Bestellliste!H82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <f>Bestellliste!A83</f>
+        <v/>
+      </c>
+      <c r="B55">
+        <f>IF(Bestellliste!C83="","",IF(Bestellliste!F83="x",4*Bestellliste!C83,Bestellliste!C83))</f>
+        <v/>
+      </c>
+      <c r="C55" s="15">
+        <f>IF(Bestellliste!D83="","",Bestellliste!D83)</f>
+        <v/>
+      </c>
+      <c r="D55" s="15">
+        <f>IF(AND(ISNUMBER(B55),ISNUMBER(C55)),B55*C55,0)</f>
+        <v/>
+      </c>
+      <c r="E55">
+        <f>IF(Bestellliste!G83="","",Bestellliste!G83)</f>
+        <v/>
+      </c>
+      <c r="F55">
+        <f>IF(Bestellliste!H83="","",Bestellliste!H83)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <f>Bestellliste!A84</f>
+        <v/>
+      </c>
+      <c r="B56">
+        <f>IF(Bestellliste!C84="","",IF(Bestellliste!F84="x",4*Bestellliste!C84,Bestellliste!C84))</f>
+        <v/>
+      </c>
+      <c r="C56" s="15">
+        <f>IF(Bestellliste!D84="","",Bestellliste!D84)</f>
+        <v/>
+      </c>
+      <c r="D56" s="15">
+        <f>IF(AND(ISNUMBER(B56),ISNUMBER(C56)),B56*C56,0)</f>
+        <v/>
+      </c>
+      <c r="E56">
+        <f>IF(Bestellliste!G84="","",Bestellliste!G84)</f>
+        <v/>
+      </c>
+      <c r="F56">
+        <f>IF(Bestellliste!H84="","",Bestellliste!H84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <f>Bestellliste!A87</f>
+        <v/>
+      </c>
+      <c r="B57">
+        <f>IF(Bestellliste!C87="","",IF(Bestellliste!F87="x",4*Bestellliste!C87,Bestellliste!C87))</f>
+        <v/>
+      </c>
+      <c r="C57" s="15">
+        <f>IF(Bestellliste!D87="","",Bestellliste!D87)</f>
+        <v/>
+      </c>
+      <c r="D57" s="15">
+        <f>IF(AND(ISNUMBER(B57),ISNUMBER(C57)),B57*C57,0)</f>
+        <v/>
+      </c>
+      <c r="E57">
+        <f>IF(Bestellliste!G87="","",Bestellliste!G87)</f>
+        <v/>
+      </c>
+      <c r="F57">
+        <f>IF(Bestellliste!H87="","",Bestellliste!H87)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <f>Bestellliste!A88</f>
+        <v/>
+      </c>
+      <c r="B58">
+        <f>IF(Bestellliste!C88="","",IF(Bestellliste!F88="x",4*Bestellliste!C88,Bestellliste!C88))</f>
+        <v/>
+      </c>
+      <c r="C58" s="15">
+        <f>IF(Bestellliste!D88="","",Bestellliste!D88)</f>
+        <v/>
+      </c>
+      <c r="D58" s="15">
+        <f>IF(AND(ISNUMBER(B58),ISNUMBER(C58)),B58*C58,0)</f>
+        <v/>
+      </c>
+      <c r="E58">
+        <f>IF(Bestellliste!G88="","",Bestellliste!G88)</f>
+        <v/>
+      </c>
+      <c r="F58">
+        <f>IF(Bestellliste!H88="","",Bestellliste!H88)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <f>Bestellliste!A89</f>
+        <v/>
+      </c>
+      <c r="B59">
+        <f>IF(Bestellliste!C89="","",IF(Bestellliste!F89="x",4*Bestellliste!C89,Bestellliste!C89))</f>
+        <v/>
+      </c>
+      <c r="C59" s="15">
+        <f>IF(Bestellliste!D89="","",Bestellliste!D89)</f>
+        <v/>
+      </c>
+      <c r="D59" s="15">
+        <f>IF(AND(ISNUMBER(B59),ISNUMBER(C59)),B59*C59,0)</f>
+        <v/>
+      </c>
+      <c r="E59">
+        <f>IF(Bestellliste!G89="","",Bestellliste!G89)</f>
+        <v/>
+      </c>
+      <c r="F59">
+        <f>IF(Bestellliste!H89="","",Bestellliste!H89)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t>Summe DOLD</t>
+        </is>
+      </c>
+      <c r="D60" s="15">
+        <f>SUM(D14:D59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Motedis</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <f>Bestellliste!A26</f>
+        <v/>
+      </c>
+      <c r="B63">
+        <f>IF(Bestellliste!C26="","",IF(Bestellliste!F26="x",4*Bestellliste!C26,Bestellliste!C26))</f>
+        <v/>
+      </c>
+      <c r="C63" s="15">
+        <f>IF(Bestellliste!D26="","",Bestellliste!D26)</f>
+        <v/>
+      </c>
+      <c r="D63" s="15">
+        <f>IF(AND(ISNUMBER(B63),ISNUMBER(C63)),B63*C63,0)</f>
+        <v/>
+      </c>
+      <c r="E63">
+        <f>IF(Bestellliste!G26="","",Bestellliste!G26)</f>
+        <v/>
+      </c>
+      <c r="F63">
+        <f>IF(Bestellliste!H26="","",Bestellliste!H26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <f>Bestellliste!A41</f>
+        <v/>
+      </c>
+      <c r="B64">
+        <f>IF(Bestellliste!C41="","",IF(Bestellliste!F41="x",4*Bestellliste!C41,Bestellliste!C41))</f>
+        <v/>
+      </c>
+      <c r="C64" s="15">
+        <f>IF(Bestellliste!D41="","",Bestellliste!D41)</f>
+        <v/>
+      </c>
+      <c r="D64" s="15">
+        <f>IF(AND(ISNUMBER(B64),ISNUMBER(C64)),B64*C64,0)</f>
+        <v/>
+      </c>
+      <c r="E64">
+        <f>IF(Bestellliste!G41="","",Bestellliste!G41)</f>
+        <v/>
+      </c>
+      <c r="F64">
+        <f>IF(Bestellliste!H41="","",Bestellliste!H41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>Summe Motedis</t>
+        </is>
+      </c>
+      <c r="D65" s="15">
+        <f>SUM(D63:D64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>Roboter-Bausatz</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <f>Bestellliste!A50</f>
+        <v/>
+      </c>
+      <c r="B68">
+        <f>IF(Bestellliste!C50="","",IF(Bestellliste!F50="x",4*Bestellliste!C50,Bestellliste!C50))</f>
+        <v/>
+      </c>
+      <c r="C68" s="15">
+        <f>IF(Bestellliste!D50="","",Bestellliste!D50)</f>
+        <v/>
+      </c>
+      <c r="D68" s="15">
+        <f>IF(AND(ISNUMBER(B68),ISNUMBER(C68)),B68*C68,0)</f>
+        <v/>
+      </c>
+      <c r="E68">
+        <f>IF(Bestellliste!G50="","",Bestellliste!G50)</f>
+        <v/>
+      </c>
+      <c r="F68">
+        <f>IF(Bestellliste!H50="","",Bestellliste!H50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <f>Bestellliste!A51</f>
+        <v/>
+      </c>
+      <c r="B69">
+        <f>IF(Bestellliste!C51="","",IF(Bestellliste!F51="x",4*Bestellliste!C51,Bestellliste!C51))</f>
+        <v/>
+      </c>
+      <c r="C69" s="15">
+        <f>IF(Bestellliste!D51="","",Bestellliste!D51)</f>
+        <v/>
+      </c>
+      <c r="D69" s="15">
+        <f>IF(AND(ISNUMBER(B69),ISNUMBER(C69)),B69*C69,0)</f>
+        <v/>
+      </c>
+      <c r="E69">
+        <f>IF(Bestellliste!G51="","",Bestellliste!G51)</f>
+        <v/>
+      </c>
+      <c r="F69">
+        <f>IF(Bestellliste!H51="","",Bestellliste!H51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>Summe Roboter-Bausatz</t>
+        </is>
+      </c>
+      <c r="D70" s="15">
+        <f>SUM(D68:D69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>StepperOnline</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <f>Bestellliste!A22</f>
+        <v/>
+      </c>
+      <c r="B73">
+        <f>IF(Bestellliste!C22="","",IF(Bestellliste!F22="x",4*Bestellliste!C22,Bestellliste!C22))</f>
+        <v/>
+      </c>
+      <c r="C73" s="15">
+        <f>IF(Bestellliste!D22="","",Bestellliste!D22)</f>
+        <v/>
+      </c>
+      <c r="D73" s="15">
+        <f>IF(AND(ISNUMBER(B73),ISNUMBER(C73)),B73*C73,0)</f>
+        <v/>
+      </c>
+      <c r="E73">
+        <f>IF(Bestellliste!G22="","",Bestellliste!G22)</f>
+        <v/>
+      </c>
+      <c r="F73">
+        <f>IF(Bestellliste!H22="","",Bestellliste!H22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <f>Bestellliste!A29</f>
+        <v/>
+      </c>
+      <c r="B74">
+        <f>IF(Bestellliste!C29="","",IF(Bestellliste!F29="x",4*Bestellliste!C29,Bestellliste!C29))</f>
+        <v/>
+      </c>
+      <c r="C74" s="15">
+        <f>IF(Bestellliste!D29="","",Bestellliste!D29)</f>
+        <v/>
+      </c>
+      <c r="D74" s="15">
+        <f>IF(AND(ISNUMBER(B74),ISNUMBER(C74)),B74*C74,0)</f>
+        <v/>
+      </c>
+      <c r="E74">
+        <f>IF(Bestellliste!G29="","",Bestellliste!G29)</f>
+        <v/>
+      </c>
+      <c r="F74">
+        <f>IF(Bestellliste!H29="","",Bestellliste!H29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <f>Bestellliste!A37</f>
+        <v/>
+      </c>
+      <c r="B75">
+        <f>IF(Bestellliste!C37="","",IF(Bestellliste!F37="x",4*Bestellliste!C37,Bestellliste!C37))</f>
+        <v/>
+      </c>
+      <c r="C75" s="15">
+        <f>IF(Bestellliste!D37="","",Bestellliste!D37)</f>
+        <v/>
+      </c>
+      <c r="D75" s="15">
+        <f>IF(AND(ISNUMBER(B75),ISNUMBER(C75)),B75*C75,0)</f>
+        <v/>
+      </c>
+      <c r="E75">
+        <f>IF(Bestellliste!G37="","",Bestellliste!G37)</f>
+        <v/>
+      </c>
+      <c r="F75">
+        <f>IF(Bestellliste!H37="","",Bestellliste!H37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>Summe StepperOnline</t>
+        </is>
+      </c>
+      <c r="D76" s="15">
+        <f>SUM(D73:D75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>Voelkner</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <f>Bestellliste!A43</f>
+        <v/>
+      </c>
+      <c r="B79">
+        <f>IF(Bestellliste!C43="","",IF(Bestellliste!F43="x",4*Bestellliste!C43,Bestellliste!C43))</f>
+        <v/>
+      </c>
+      <c r="C79" s="15">
+        <f>IF(Bestellliste!D43="","",Bestellliste!D43)</f>
+        <v/>
+      </c>
+      <c r="D79" s="15">
+        <f>IF(AND(ISNUMBER(B79),ISNUMBER(C79)),B79*C79,0)</f>
+        <v/>
+      </c>
+      <c r="E79">
+        <f>IF(Bestellliste!G43="","",Bestellliste!G43)</f>
+        <v/>
+      </c>
+      <c r="F79">
+        <f>IF(Bestellliste!H43="","",Bestellliste!H43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>Summe Voelkner</t>
+        </is>
+      </c>
+      <c r="D80" s="15">
+        <f>SUM(D79:D79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>Werkstatt</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <f>Bestellliste!A16</f>
+        <v/>
+      </c>
+      <c r="B83">
+        <f>IF(Bestellliste!C16="","",IF(Bestellliste!F16="x",4*Bestellliste!C16,Bestellliste!C16))</f>
+        <v/>
+      </c>
+      <c r="C83" s="15">
+        <f>IF(Bestellliste!D16="","",Bestellliste!D16)</f>
+        <v/>
+      </c>
+      <c r="D83" s="15">
+        <f>IF(AND(ISNUMBER(B83),ISNUMBER(C83)),B83*C83,0)</f>
+        <v/>
+      </c>
+      <c r="E83">
+        <f>IF(Bestellliste!G16="","",Bestellliste!G16)</f>
+        <v/>
+      </c>
+      <c r="F83">
+        <f>IF(Bestellliste!H16="","",Bestellliste!H16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <f>Bestellliste!A28</f>
+        <v/>
+      </c>
+      <c r="B84">
+        <f>IF(Bestellliste!C28="","",IF(Bestellliste!F28="x",4*Bestellliste!C28,Bestellliste!C28))</f>
+        <v/>
+      </c>
+      <c r="C84" s="15">
+        <f>IF(Bestellliste!D28="","",Bestellliste!D28)</f>
+        <v/>
+      </c>
+      <c r="D84" s="15">
+        <f>IF(AND(ISNUMBER(B84),ISNUMBER(C84)),B84*C84,0)</f>
+        <v/>
+      </c>
+      <c r="E84">
+        <f>IF(Bestellliste!G28="","",Bestellliste!G28)</f>
+        <v/>
+      </c>
+      <c r="F84">
+        <f>IF(Bestellliste!H28="","",Bestellliste!H28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="16" t="inlineStr">
+        <is>
+          <t>Summe Werkstatt</t>
+        </is>
+      </c>
+      <c r="D85" s="15">
+        <f>SUM(D83:D84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>igus</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <f>Bestellliste!A56</f>
+        <v/>
+      </c>
+      <c r="B88">
+        <f>IF(Bestellliste!C56="","",IF(Bestellliste!F56="x",4*Bestellliste!C56,Bestellliste!C56))</f>
+        <v/>
+      </c>
+      <c r="C88" s="15">
+        <f>IF(Bestellliste!D56="","",Bestellliste!D56)</f>
+        <v/>
+      </c>
+      <c r="D88" s="15">
+        <f>IF(AND(ISNUMBER(B88),ISNUMBER(C88)),B88*C88,0)</f>
+        <v/>
+      </c>
+      <c r="E88">
+        <f>IF(Bestellliste!G56="","",Bestellliste!G56)</f>
+        <v/>
+      </c>
+      <c r="F88">
+        <f>IF(Bestellliste!H56="","",Bestellliste!H56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <f>Bestellliste!A57</f>
+        <v/>
+      </c>
+      <c r="B89">
+        <f>IF(Bestellliste!C57="","",IF(Bestellliste!F57="x",4*Bestellliste!C57,Bestellliste!C57))</f>
+        <v/>
+      </c>
+      <c r="C89" s="15">
+        <f>IF(Bestellliste!D57="","",Bestellliste!D57)</f>
+        <v/>
+      </c>
+      <c r="D89" s="15">
+        <f>IF(AND(ISNUMBER(B89),ISNUMBER(C89)),B89*C89,0)</f>
+        <v/>
+      </c>
+      <c r="E89">
+        <f>IF(Bestellliste!G57="","",Bestellliste!G57)</f>
+        <v/>
+      </c>
+      <c r="F89">
+        <f>IF(Bestellliste!H57="","",Bestellliste!H57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="16" t="inlineStr">
+        <is>
+          <t>Summe igus</t>
+        </is>
+      </c>
+      <c r="D90" s="15">
+        <f>SUM(D88:D89)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <t>ohne Shop (noch offen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <f>Bestellliste!A15</f>
+        <v/>
+      </c>
+      <c r="B93">
+        <f>IF(Bestellliste!C15="","",IF(Bestellliste!F15="x",4*Bestellliste!C15,Bestellliste!C15))</f>
+        <v/>
+      </c>
+      <c r="C93" s="15">
+        <f>IF(Bestellliste!D15="","",Bestellliste!D15)</f>
+        <v/>
+      </c>
+      <c r="D93" s="15">
+        <f>IF(AND(ISNUMBER(B93),ISNUMBER(C93)),B93*C93,0)</f>
+        <v/>
+      </c>
+      <c r="E93">
+        <f>IF(Bestellliste!G15="","",Bestellliste!G15)</f>
+        <v/>
+      </c>
+      <c r="F93">
+        <f>IF(Bestellliste!H15="","",Bestellliste!H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
+        <f>Bestellliste!A47</f>
+        <v/>
+      </c>
+      <c r="B94">
+        <f>IF(Bestellliste!C47="","",IF(Bestellliste!F47="x",4*Bestellliste!C47,Bestellliste!C47))</f>
+        <v/>
+      </c>
+      <c r="C94" s="15">
+        <f>IF(Bestellliste!D47="","",Bestellliste!D47)</f>
+        <v/>
+      </c>
+      <c r="D94" s="15">
+        <f>IF(AND(ISNUMBER(B94),ISNUMBER(C94)),B94*C94,0)</f>
+        <v/>
+      </c>
+      <c r="E94">
+        <f>IF(Bestellliste!G47="","",Bestellliste!G47)</f>
+        <v/>
+      </c>
+      <c r="F94">
+        <f>IF(Bestellliste!H47="","",Bestellliste!H47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95">
+        <f>Bestellliste!A53</f>
+        <v/>
+      </c>
+      <c r="B95">
+        <f>IF(Bestellliste!C53="","",IF(Bestellliste!F53="x",4*Bestellliste!C53,Bestellliste!C53))</f>
+        <v/>
+      </c>
+      <c r="C95" s="15">
+        <f>IF(Bestellliste!D53="","",Bestellliste!D53)</f>
+        <v/>
+      </c>
+      <c r="D95" s="15">
+        <f>IF(AND(ISNUMBER(B95),ISNUMBER(C95)),B95*C95,0)</f>
+        <v/>
+      </c>
+      <c r="E95">
+        <f>IF(Bestellliste!G53="","",Bestellliste!G53)</f>
+        <v/>
+      </c>
+      <c r="F95">
+        <f>IF(Bestellliste!H53="","",Bestellliste!H53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <f>Bestellliste!A54</f>
+        <v/>
+      </c>
+      <c r="B96">
+        <f>IF(Bestellliste!C54="","",IF(Bestellliste!F54="x",4*Bestellliste!C54,Bestellliste!C54))</f>
+        <v/>
+      </c>
+      <c r="C96" s="15">
+        <f>IF(Bestellliste!D54="","",Bestellliste!D54)</f>
+        <v/>
+      </c>
+      <c r="D96" s="15">
+        <f>IF(AND(ISNUMBER(B96),ISNUMBER(C96)),B96*C96,0)</f>
+        <v/>
+      </c>
+      <c r="E96">
+        <f>IF(Bestellliste!G54="","",Bestellliste!G54)</f>
+        <v/>
+      </c>
+      <c r="F96">
+        <f>IF(Bestellliste!H54="","",Bestellliste!H54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <f>Bestellliste!A55</f>
+        <v/>
+      </c>
+      <c r="B97">
+        <f>IF(Bestellliste!C55="","",IF(Bestellliste!F55="x",4*Bestellliste!C55,Bestellliste!C55))</f>
+        <v/>
+      </c>
+      <c r="C97" s="15">
+        <f>IF(Bestellliste!D55="","",Bestellliste!D55)</f>
+        <v/>
+      </c>
+      <c r="D97" s="15">
+        <f>IF(AND(ISNUMBER(B97),ISNUMBER(C97)),B97*C97,0)</f>
+        <v/>
+      </c>
+      <c r="E97">
+        <f>IF(Bestellliste!G55="","",Bestellliste!G55)</f>
+        <v/>
+      </c>
+      <c r="F97">
+        <f>IF(Bestellliste!H55="","",Bestellliste!H55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <f>Bestellliste!A58</f>
+        <v/>
+      </c>
+      <c r="B98">
+        <f>IF(Bestellliste!C58="","",IF(Bestellliste!F58="x",4*Bestellliste!C58,Bestellliste!C58))</f>
+        <v/>
+      </c>
+      <c r="C98" s="15">
+        <f>IF(Bestellliste!D58="","",Bestellliste!D58)</f>
+        <v/>
+      </c>
+      <c r="D98" s="15">
+        <f>IF(AND(ISNUMBER(B98),ISNUMBER(C98)),B98*C98,0)</f>
+        <v/>
+      </c>
+      <c r="E98">
+        <f>IF(Bestellliste!G58="","",Bestellliste!G58)</f>
+        <v/>
+      </c>
+      <c r="F98">
+        <f>IF(Bestellliste!H58="","",Bestellliste!H58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <f>Bestellliste!A59</f>
+        <v/>
+      </c>
+      <c r="B99">
+        <f>IF(Bestellliste!C59="","",IF(Bestellliste!F59="x",4*Bestellliste!C59,Bestellliste!C59))</f>
+        <v/>
+      </c>
+      <c r="C99" s="15">
+        <f>IF(Bestellliste!D59="","",Bestellliste!D59)</f>
+        <v/>
+      </c>
+      <c r="D99" s="15">
+        <f>IF(AND(ISNUMBER(B99),ISNUMBER(C99)),B99*C99,0)</f>
+        <v/>
+      </c>
+      <c r="E99">
+        <f>IF(Bestellliste!G59="","",Bestellliste!G59)</f>
+        <v/>
+      </c>
+      <c r="F99">
+        <f>IF(Bestellliste!H59="","",Bestellliste!H59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <f>Bestellliste!A85</f>
+        <v/>
+      </c>
+      <c r="B100">
+        <f>IF(Bestellliste!C85="","",IF(Bestellliste!F85="x",4*Bestellliste!C85,Bestellliste!C85))</f>
+        <v/>
+      </c>
+      <c r="C100" s="15">
+        <f>IF(Bestellliste!D85="","",Bestellliste!D85)</f>
+        <v/>
+      </c>
+      <c r="D100" s="15">
+        <f>IF(AND(ISNUMBER(B100),ISNUMBER(C100)),B100*C100,0)</f>
+        <v/>
+      </c>
+      <c r="E100">
+        <f>IF(Bestellliste!G85="","",Bestellliste!G85)</f>
+        <v/>
+      </c>
+      <c r="F100">
+        <f>IF(Bestellliste!H85="","",Bestellliste!H85)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <f>Bestellliste!A86</f>
+        <v/>
+      </c>
+      <c r="B101">
+        <f>IF(Bestellliste!C86="","",IF(Bestellliste!F86="x",4*Bestellliste!C86,Bestellliste!C86))</f>
+        <v/>
+      </c>
+      <c r="C101" s="15">
+        <f>IF(Bestellliste!D86="","",Bestellliste!D86)</f>
+        <v/>
+      </c>
+      <c r="D101" s="15">
+        <f>IF(AND(ISNUMBER(B101),ISNUMBER(C101)),B101*C101,0)</f>
+        <v/>
+      </c>
+      <c r="E101">
+        <f>IF(Bestellliste!G86="","",Bestellliste!G86)</f>
+        <v/>
+      </c>
+      <c r="F101">
+        <f>IF(Bestellliste!H86="","",Bestellliste!H86)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="16" t="inlineStr">
+        <is>
+          <t>Summe ohne Shop (noch offen)</t>
+        </is>
+      </c>
+      <c r="D102" s="15">
+        <f>SUM(D93:D101)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>Gesamt Vollausbau inkl. MwSt.</t>
+        </is>
+      </c>
+      <c r="D104" s="17">
+        <f>D11+D60+D65+D70+D76+D80+D85+D90+D102</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Werte sind mit dem Blatt „Bestellliste“ verknüpft; Status dort in Spalte H pflegen.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>